<commit_message>
Clarify security selection and Decision Log guidance
</commit_message>
<xml_diff>
--- a/files/BUS331_InvProject_SecuritySelection_Template.xlsx
+++ b/files/BUS331_InvProject_SecuritySelection_Template.xlsx
@@ -7,7 +7,7 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client 1" sheetId="3" r:id="rId9"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client 2" sheetId="4" r:id="rId10"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client 3" sheetId="5" r:id="rId11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ISSUER CHECK" sheetId="6" r:id="rId12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REALITY CHECK" sheetId="11" r:id="rId12"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EVIDENCE LOG" sheetId="7" r:id="rId13"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESEARCH GUIDE" sheetId="8" r:id="rId14"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FINAL SCORECARDS" sheetId="9" r:id="rId15"/>
@@ -3360,7 +3360,7 @@
     <x:numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="39">
+  <x:fonts count="40">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -3575,6 +3575,11 @@
       <x:b/>
       <x:sz val="10"/>
       <x:color rgb="FF102238"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF008000"/>
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
@@ -4231,7 +4236,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="36">
+  <x:borders count="38">
     <x:border/>
     <x:border>
       <x:bottom style="medium">
@@ -4573,6 +4578,31 @@
         <x:color rgb="FFD9E2EA"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2EA"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE6EDF2"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2EA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2EA"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE6EDF2"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2EA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2EA"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="6">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -4582,7 +4612,7 @@
     <x:xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1710">
+  <x:cellXfs count="1718">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="14" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -8660,6 +8690,42 @@
     <x:xf numFmtId="0" fontId="29" fillId="119" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="119" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="119" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="119" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="119" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="119" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="119" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="119" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="119" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="119" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="119" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="119" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="119" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="29" fillId="129" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
@@ -8678,22 +8744,19 @@
     <x:xf numFmtId="0" fontId="29" fillId="129" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="164" fontId="29" fillId="119" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="29" fillId="119" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="29" fillId="119" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="29" fillId="119" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="29" fillId="119" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="29" fillId="119" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="164" fontId="39" fillId="119" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="39" fillId="119" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="29" fillId="121" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="29" fillId="121" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="29" fillId="121" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="130" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -8703,15 +8766,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="30" fillId="130" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="29" fillId="121" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="29" fillId="121" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="29" fillId="121" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="6">
@@ -9281,7 +9335,7 @@
     <x:row r="6" ht="45.75" customHeight="1">
       <x:c r="A6" s="86"/>
       <x:c r="B6" s="90" t="str">
-        <x:v>Use the client tabs for candidate work, FINAL SCORECARDS for the 8–10 final holdings per client, RISK &amp; HEDGE for the residual-risk conclusion, ISSUER CHECK only where required, and EVIDENCE LOG for licensed-source research. Never exceed 10 holdings; do not fill a slot without a purpose.</x:v>
+        <x:v>Use the client tabs for the 8–10 holdings currently proposed for each client, FINAL SCORECARDS for the authoritative Phase 2 final-holding record, REALITY CHECK to validate each proposed final holding and any conditional direct-security add-on, RISK &amp; HEDGE for the residual-risk conclusion, and EVIDENCE LOG for licensed-source research. Never exceed 10 holdings; do not fill a slot without a purpose.</x:v>
       </x:c>
       <x:c r="C6" s="90"/>
       <x:c r="D6" s="86"/>
@@ -9324,7 +9378,7 @@
     <x:row r="9" ht="45.75" customHeight="1">
       <x:c r="A9" s="86"/>
       <x:c r="B9" s="90" t="str">
-        <x:v>Your Phase 1 market view, client IPS, unresolved information gaps, and downstream guardrails must be approved before security research begins. Every candidate and Issuer Reality Check must trace to that mandate; the macro filter on each client tab must pass before selection.</x:v>
+        <x:v>Your Phase 1 market view, client IPS, unresolved information gaps, and downstream guardrails must be approved before security research begins. Every proposed holding and Holding &amp; Exposure Reality Check must trace to that mandate; the macro filter on each client tab must pass before selection.</x:v>
       </x:c>
       <x:c r="C9" s="90"/>
       <x:c r="D9" s="86"/>
@@ -9352,7 +9406,7 @@
     <x:row r="11" ht="34" customHeight="1">
       <x:c r="A11" s="86"/>
       <x:c r="B11" s="89" t="str">
-        <x:v>  Section 1 — Candidate Research and Final Scorecards</x:v>
+        <x:v>  Section 1 — Proposed Final Portfolios and Final Scorecards</x:v>
       </x:c>
       <x:c r="C11" s="86"/>
       <x:c r="D11" s="86"/>
@@ -9367,7 +9421,7 @@
     <x:row r="12" ht="45.75" customHeight="1">
       <x:c r="A12" s="86"/>
       <x:c r="B12" s="90" t="str">
-        <x:v>Use the client tabs for focused candidate research. Compare realistic alternatives concisely, then record only the 8–10 final holdings per client in FINAL SCORECARDS. Never exceed 10, do not fill an unused slot, keep funds and ETFs primary, and limit individual securities to two or three total.</x:v>
+        <x:v>Use each client tab for the 8–10 final holdings the team currently intends to recommend and any selective decision notes that matter. Record the authoritative Phase 2 final holdings in FINAL SCORECARDS. Never exceed 10, do not fill an unused slot, keep funds and ETFs primary, and limit direct individual securities to two or three total.</x:v>
       </x:c>
       <x:c r="C12" s="90"/>
       <x:c r="D12" s="86"/>
@@ -9438,7 +9492,7 @@
     <x:row r="17" ht="34" customHeight="1">
       <x:c r="A17" s="86"/>
       <x:c r="B17" s="89" t="str">
-        <x:v>  Section 3 — Final-Holding Evidence and Decision Log</x:v>
+        <x:v>  Section 3 — Final-Holding Evidence and Project Decision Trail</x:v>
       </x:c>
       <x:c r="C17" s="86"/>
       <x:c r="D17" s="86"/>
@@ -9453,7 +9507,7 @@
     <x:row r="18" ht="45.75" customHeight="1">
       <x:c r="A18" s="86"/>
       <x:c r="B18" s="90" t="str">
-        <x:v>Complete one concise scorecard for every final holding and record the recommendation, strongest alternative rejected, and key trade-off in the Analyst Decision Log. Full analysis is not required for every screened candidate.</x:v>
+        <x:v>Complete one concise Holding &amp; Exposure Reality Check row for every proposed final holding. Use FINAL SCORECARDS as the authoritative Phase 2 final-holding record; continue consequential recommendations, alternatives rejected, trade-offs, verifications, and approvals in the project-wide Analyst Decision Log.</x:v>
       </x:c>
       <x:c r="C18" s="90"/>
       <x:c r="D18" s="86"/>
@@ -10277,7 +10331,7 @@
     <x:row r="8" ht="7.5" customHeight="1"/>
     <x:row r="9" ht="19.5" customHeight="1">
       <x:c r="A9" s="5" t="str">
-        <x:v>  SECTION 1 — FOCUSED CANDIDATE RESEARCH TABLE</x:v>
+        <x:v>  SECTION 1 — PROPOSED FINAL PORTFOLIO — RESEARCH &amp; ALLOCATION</x:v>
       </x:c>
       <x:c r="B9" s="5"/>
       <x:c r="C9" s="5"/>
@@ -10292,9 +10346,9 @@
       <x:c r="L9" s="5"/>
       <x:c r="M9" s="5"/>
     </x:row>
-    <x:row r="10" ht="30" customHeight="1">
+    <x:row r="10" ht="44" customHeight="1">
       <x:c r="A10" s="8" t="str">
-        <x:v>Use this tab for candidate research and calculations. Record the 8–10 final holdings in FINAL SCORECARDS; never exceed 10, do not fill every slot, keep funds/ETFs primary, and limit individual securities to two or three total.</x:v>
+        <x:v>Enter the 8–10 final holdings the team currently intends to recommend for this client. Never exceed 10, do not fill an unused slot, keep funds and ETFs primary, and limit direct individual securities to two or three total. Record the authoritative Phase 2 final holdings in FINAL SCORECARDS.</x:v>
       </x:c>
       <x:c r="B10" s="8"/>
       <x:c r="C10" s="8"/>
@@ -10338,7 +10392,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="K11" s="27" t="str">
-        <x:v>Candidate Note
+        <x:v>Decision Note
 Ref #</x:v>
       </x:c>
       <x:c r="L11" s="27" t="s">
@@ -10800,9 +10854,9 @@
       <x:c r="L40" s="7"/>
     </x:row>
     <x:row r="41" ht="9.75" customHeight="1"/>
-    <x:row r="42" ht="19.5" customHeight="1">
+    <x:row r="42" ht="30" customHeight="1">
       <x:c r="A42" s="5" t="str">
-        <x:v>  SECTION 3 — CANDIDATE NOTES (NOT FINAL SCORECARDS)</x:v>
+        <x:v>  SECTION 3 — OPTIONAL DECISION NOTES — SELECTED HOLDINGS OR REJECTED ALTERNATIVES</x:v>
       </x:c>
       <x:c r="B42" s="5"/>
       <x:c r="C42" s="5"/>
@@ -10817,9 +10871,9 @@
       <x:c r="L42" s="5"/>
       <x:c r="M42" s="5"/>
     </x:row>
-    <x:row r="43" ht="30" customHeight="1">
+    <x:row r="43" ht="48" customHeight="1">
       <x:c r="A43" s="8" t="str">
-        <x:v>Use a brief candidate note only when it materially supports a final Select or Reject decision. Do not complete one block for every screened name. FINAL SCORECARDS and the Analyst Decision Log are the authoritative final records.</x:v>
+        <x:v>Use these selective, optional notes only when they support a consequential Select or Reject decision. They are not a second candidate list and are not required for every screened name. FINAL SCORECARDS are the authoritative Phase 2 final-holding record; the Analyst Decision Log is the continuing, project-wide decision and audit trail.</x:v>
       </x:c>
       <x:c r="B43" s="8"/>
       <x:c r="C43" s="8"/>
@@ -10836,7 +10890,7 @@
     </x:row>
     <x:row r="44" ht="19.5" customHeight="1">
       <x:c r="A44" s="73" t="str">
-        <x:v>  Candidate Note #1</x:v>
+        <x:v>  Optional Decision Note #1</x:v>
       </x:c>
       <x:c r="B44" s="73"/>
       <x:c r="C44" s="73"/>
@@ -10966,7 +11020,7 @@
     <x:row r="52" ht="6" customHeight="1"/>
     <x:row r="53" ht="19.5" customHeight="1">
       <x:c r="A53" s="73" t="str">
-        <x:v>  Candidate Note #2</x:v>
+        <x:v>  Optional Decision Note #2</x:v>
       </x:c>
       <x:c r="B53" s="73"/>
       <x:c r="C53" s="73"/>
@@ -11096,7 +11150,7 @@
     <x:row r="61" ht="6" customHeight="1"/>
     <x:row r="62" ht="19.5" customHeight="1">
       <x:c r="A62" s="73" t="str">
-        <x:v>  Candidate Note #3</x:v>
+        <x:v>  Optional Decision Note #3</x:v>
       </x:c>
       <x:c r="B62" s="73"/>
       <x:c r="C62" s="73"/>
@@ -11226,7 +11280,7 @@
     <x:row r="70" ht="6" customHeight="1"/>
     <x:row r="71" ht="19.5" customHeight="1">
       <x:c r="A71" s="73" t="str">
-        <x:v>  Candidate Note #4</x:v>
+        <x:v>  Optional Decision Note #4</x:v>
       </x:c>
       <x:c r="B71" s="73"/>
       <x:c r="C71" s="73"/>
@@ -11356,7 +11410,7 @@
     <x:row r="79" ht="6" customHeight="1"/>
     <x:row r="80" ht="19.5" customHeight="1">
       <x:c r="A80" s="73" t="str">
-        <x:v>  Candidate Note #5</x:v>
+        <x:v>  Optional Decision Note #5</x:v>
       </x:c>
       <x:c r="B80" s="73"/>
       <x:c r="C80" s="73"/>
@@ -11484,9 +11538,9 @@
       <x:c r="M87" s="7"/>
     </x:row>
     <x:row r="88" ht="6" customHeight="1"/>
-    <x:row r="89" ht="27.75" customHeight="1">
+    <x:row r="89" ht="32" customHeight="1">
       <x:c r="A89" s="74" t="str">
-        <x:v>  ▲ Do not add a note block unless it materially supports a final Select or Reject decision. Full analysis is not required for every screened candidate.</x:v>
+        <x:v>  ▲ Use a note only for a consequential Select or Reject decision. These notes are optional support—not a second candidate list or a required record for every screened name.</x:v>
       </x:c>
       <x:c r="B89" s="74"/>
       <x:c r="C89" s="74"/>
@@ -11835,7 +11889,7 @@
     <x:row r="8" ht="7.5" customHeight="1"/>
     <x:row r="9" ht="19.5" customHeight="1">
       <x:c r="A9" s="5" t="str">
-        <x:v>  SECTION 1 — FOCUSED CANDIDATE RESEARCH TABLE</x:v>
+        <x:v>  SECTION 1 — PROPOSED FINAL PORTFOLIO — RESEARCH &amp; ALLOCATION</x:v>
       </x:c>
       <x:c r="B9" s="5"/>
       <x:c r="C9" s="5"/>
@@ -11850,9 +11904,9 @@
       <x:c r="L9" s="5"/>
       <x:c r="M9" s="5"/>
     </x:row>
-    <x:row r="10" ht="30" customHeight="1">
+    <x:row r="10" ht="44" customHeight="1">
       <x:c r="A10" s="8" t="str">
-        <x:v>Use this tab for candidate research and calculations. Record the 8–10 final holdings in FINAL SCORECARDS; never exceed 10, do not fill every slot, keep funds/ETFs primary, and limit individual securities to two or three total.</x:v>
+        <x:v>Enter the 8–10 final holdings the team currently intends to recommend for this client. Never exceed 10, do not fill an unused slot, keep funds and ETFs primary, and limit direct individual securities to two or three total. Record the authoritative Phase 2 final holdings in FINAL SCORECARDS.</x:v>
       </x:c>
       <x:c r="B10" s="8"/>
       <x:c r="C10" s="8"/>
@@ -11896,7 +11950,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="K11" s="27" t="str">
-        <x:v>Candidate Note
+        <x:v>Decision Note
 Ref #</x:v>
       </x:c>
       <x:c r="L11" s="27" t="s">
@@ -12358,9 +12412,9 @@
       <x:c r="L40" s="7"/>
     </x:row>
     <x:row r="41" ht="9.75" customHeight="1"/>
-    <x:row r="42" ht="19.5" customHeight="1">
+    <x:row r="42" ht="30" customHeight="1">
       <x:c r="A42" s="5" t="str">
-        <x:v>  SECTION 3 — CANDIDATE NOTES (NOT FINAL SCORECARDS)</x:v>
+        <x:v>  SECTION 3 — OPTIONAL DECISION NOTES — SELECTED HOLDINGS OR REJECTED ALTERNATIVES</x:v>
       </x:c>
       <x:c r="B42" s="5"/>
       <x:c r="C42" s="5"/>
@@ -12375,9 +12429,9 @@
       <x:c r="L42" s="5"/>
       <x:c r="M42" s="5"/>
     </x:row>
-    <x:row r="43" ht="30" customHeight="1">
+    <x:row r="43" ht="48" customHeight="1">
       <x:c r="A43" s="8" t="str">
-        <x:v>Use a brief candidate note only when it materially supports a final Select or Reject decision. Do not complete one block for every screened name. FINAL SCORECARDS and the Analyst Decision Log are the authoritative final records.</x:v>
+        <x:v>Use these selective, optional notes only when they support a consequential Select or Reject decision. They are not a second candidate list and are not required for every screened name. FINAL SCORECARDS are the authoritative Phase 2 final-holding record; the Analyst Decision Log is the continuing, project-wide decision and audit trail.</x:v>
       </x:c>
       <x:c r="B43" s="8"/>
       <x:c r="C43" s="8"/>
@@ -12394,7 +12448,7 @@
     </x:row>
     <x:row r="44" ht="19.5" customHeight="1">
       <x:c r="A44" s="73" t="str">
-        <x:v>  Candidate Note #1</x:v>
+        <x:v>  Optional Decision Note #1</x:v>
       </x:c>
       <x:c r="B44" s="73"/>
       <x:c r="C44" s="73"/>
@@ -12524,7 +12578,7 @@
     <x:row r="52" ht="6" customHeight="1"/>
     <x:row r="53" ht="19.5" customHeight="1">
       <x:c r="A53" s="73" t="str">
-        <x:v>  Candidate Note #2</x:v>
+        <x:v>  Optional Decision Note #2</x:v>
       </x:c>
       <x:c r="B53" s="73"/>
       <x:c r="C53" s="73"/>
@@ -12654,7 +12708,7 @@
     <x:row r="61" ht="6" customHeight="1"/>
     <x:row r="62" ht="19.5" customHeight="1">
       <x:c r="A62" s="73" t="str">
-        <x:v>  Candidate Note #3</x:v>
+        <x:v>  Optional Decision Note #3</x:v>
       </x:c>
       <x:c r="B62" s="73"/>
       <x:c r="C62" s="73"/>
@@ -12784,7 +12838,7 @@
     <x:row r="70" ht="6" customHeight="1"/>
     <x:row r="71" ht="19.5" customHeight="1">
       <x:c r="A71" s="73" t="str">
-        <x:v>  Candidate Note #4</x:v>
+        <x:v>  Optional Decision Note #4</x:v>
       </x:c>
       <x:c r="B71" s="73"/>
       <x:c r="C71" s="73"/>
@@ -12914,7 +12968,7 @@
     <x:row r="79" ht="6" customHeight="1"/>
     <x:row r="80" ht="19.5" customHeight="1">
       <x:c r="A80" s="73" t="str">
-        <x:v>  Candidate Note #5</x:v>
+        <x:v>  Optional Decision Note #5</x:v>
       </x:c>
       <x:c r="B80" s="73"/>
       <x:c r="C80" s="73"/>
@@ -13042,9 +13096,9 @@
       <x:c r="M87" s="7"/>
     </x:row>
     <x:row r="88" ht="6" customHeight="1"/>
-    <x:row r="89" ht="27.75" customHeight="1">
+    <x:row r="89" ht="32" customHeight="1">
       <x:c r="A89" s="74" t="str">
-        <x:v>  ▲ Do not add a note block unless it materially supports a final Select or Reject decision. Full analysis is not required for every screened candidate.</x:v>
+        <x:v>  ▲ Use a note only for a consequential Select or Reject decision. These notes are optional support—not a second candidate list or a required record for every screened name.</x:v>
       </x:c>
       <x:c r="B89" s="74"/>
       <x:c r="C89" s="74"/>
@@ -13393,7 +13447,7 @@
     <x:row r="8" ht="7.5" customHeight="1"/>
     <x:row r="9" ht="19.5" customHeight="1">
       <x:c r="A9" s="5" t="str">
-        <x:v>  SECTION 1 — FOCUSED CANDIDATE RESEARCH TABLE</x:v>
+        <x:v>  SECTION 1 — PROPOSED FINAL PORTFOLIO — RESEARCH &amp; ALLOCATION</x:v>
       </x:c>
       <x:c r="B9" s="5"/>
       <x:c r="C9" s="5"/>
@@ -13408,9 +13462,9 @@
       <x:c r="L9" s="5"/>
       <x:c r="M9" s="5"/>
     </x:row>
-    <x:row r="10" ht="30" customHeight="1">
+    <x:row r="10" ht="44" customHeight="1">
       <x:c r="A10" s="8" t="str">
-        <x:v>Use this tab for candidate research and calculations. Record the 8–10 final holdings in FINAL SCORECARDS; never exceed 10, do not fill every slot, keep funds/ETFs primary, and limit individual securities to two or three total.</x:v>
+        <x:v>Enter the 8–10 final holdings the team currently intends to recommend for this client. Never exceed 10, do not fill an unused slot, keep funds and ETFs primary, and limit direct individual securities to two or three total. Record the authoritative Phase 2 final holdings in FINAL SCORECARDS.</x:v>
       </x:c>
       <x:c r="B10" s="8"/>
       <x:c r="C10" s="8"/>
@@ -13454,7 +13508,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="K11" s="27" t="str">
-        <x:v>Candidate Note
+        <x:v>Decision Note
 Ref #</x:v>
       </x:c>
       <x:c r="L11" s="27" t="s">
@@ -13916,9 +13970,9 @@
       <x:c r="L40" s="7"/>
     </x:row>
     <x:row r="41" ht="9.75" customHeight="1"/>
-    <x:row r="42" ht="19.5" customHeight="1">
+    <x:row r="42" ht="30" customHeight="1">
       <x:c r="A42" s="5" t="str">
-        <x:v>  SECTION 3 — CANDIDATE NOTES (NOT FINAL SCORECARDS)</x:v>
+        <x:v>  SECTION 3 — OPTIONAL DECISION NOTES — SELECTED HOLDINGS OR REJECTED ALTERNATIVES</x:v>
       </x:c>
       <x:c r="B42" s="5"/>
       <x:c r="C42" s="5"/>
@@ -13933,9 +13987,9 @@
       <x:c r="L42" s="5"/>
       <x:c r="M42" s="5"/>
     </x:row>
-    <x:row r="43" ht="30" customHeight="1">
+    <x:row r="43" ht="48" customHeight="1">
       <x:c r="A43" s="8" t="str">
-        <x:v>Use a brief candidate note only when it materially supports a final Select or Reject decision. Do not complete one block for every screened name. FINAL SCORECARDS and the Analyst Decision Log are the authoritative final records.</x:v>
+        <x:v>Use these selective, optional notes only when they support a consequential Select or Reject decision. They are not a second candidate list and are not required for every screened name. FINAL SCORECARDS are the authoritative Phase 2 final-holding record; the Analyst Decision Log is the continuing, project-wide decision and audit trail.</x:v>
       </x:c>
       <x:c r="B43" s="8"/>
       <x:c r="C43" s="8"/>
@@ -13952,7 +14006,7 @@
     </x:row>
     <x:row r="44" ht="19.5" customHeight="1">
       <x:c r="A44" s="73" t="str">
-        <x:v>  Candidate Note #1</x:v>
+        <x:v>  Optional Decision Note #1</x:v>
       </x:c>
       <x:c r="B44" s="73"/>
       <x:c r="C44" s="73"/>
@@ -14082,7 +14136,7 @@
     <x:row r="52" ht="6" customHeight="1"/>
     <x:row r="53" ht="19.5" customHeight="1">
       <x:c r="A53" s="73" t="str">
-        <x:v>  Candidate Note #2</x:v>
+        <x:v>  Optional Decision Note #2</x:v>
       </x:c>
       <x:c r="B53" s="73"/>
       <x:c r="C53" s="73"/>
@@ -14212,7 +14266,7 @@
     <x:row r="61" ht="6" customHeight="1"/>
     <x:row r="62" ht="19.5" customHeight="1">
       <x:c r="A62" s="73" t="str">
-        <x:v>  Candidate Note #3</x:v>
+        <x:v>  Optional Decision Note #3</x:v>
       </x:c>
       <x:c r="B62" s="73"/>
       <x:c r="C62" s="73"/>
@@ -14342,7 +14396,7 @@
     <x:row r="70" ht="6" customHeight="1"/>
     <x:row r="71" ht="19.5" customHeight="1">
       <x:c r="A71" s="73" t="str">
-        <x:v>  Candidate Note #4</x:v>
+        <x:v>  Optional Decision Note #4</x:v>
       </x:c>
       <x:c r="B71" s="73"/>
       <x:c r="C71" s="73"/>
@@ -14472,7 +14526,7 @@
     <x:row r="79" ht="6" customHeight="1"/>
     <x:row r="80" ht="19.5" customHeight="1">
       <x:c r="A80" s="73" t="str">
-        <x:v>  Candidate Note #5</x:v>
+        <x:v>  Optional Decision Note #5</x:v>
       </x:c>
       <x:c r="B80" s="73"/>
       <x:c r="C80" s="73"/>
@@ -14600,9 +14654,9 @@
       <x:c r="M87" s="7"/>
     </x:row>
     <x:row r="88" ht="6" customHeight="1"/>
-    <x:row r="89" ht="27.75" customHeight="1">
+    <x:row r="89" ht="32" customHeight="1">
       <x:c r="A89" s="74" t="str">
-        <x:v>  ▲ Do not add a note block unless it materially supports a final Select or Reject decision. Full analysis is not required for every screened candidate.</x:v>
+        <x:v>  ▲ Use a note only for a consequential Select or Reject decision. These notes are optional support—not a second candidate list or a required record for every screened name.</x:v>
       </x:c>
       <x:c r="B89" s="74"/>
       <x:c r="C89" s="74"/>
@@ -14855,41 +14909,34 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
-    <x:col min="2" max="3" width="18" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="8" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
-    <x:col min="9" max="10" width="24" customWidth="1"/>
-    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
-    <x:col min="12" max="13" width="18" customWidth="1"/>
-    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
-    <x:col min="15" max="16" width="18" customWidth="1"/>
-    <x:col min="17" max="17" width="28" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="26" hidden="0" customWidth="1"/>
-    <x:col min="20" max="21" width="22" customWidth="1"/>
-    <x:col min="22" max="22" width="20" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="17" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="18" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="22" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="27" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="25" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="23" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="27" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="14" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="30" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="29" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="22" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="20" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="17" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="1481" t="str">
-        <x:v>BUS 331 — Issuer Reality Check</x:v>
+        <x:v>BUS 331 — Holding &amp; Exposure Reality Check</x:v>
       </x:c>
       <x:c r="B1" s="1481"/>
       <x:c r="C1" s="1481"/>
@@ -14911,12 +14958,10 @@
       <x:c r="S1" s="1481"/>
       <x:c r="T1" s="1481"/>
       <x:c r="U1" s="1481"/>
-      <x:c r="V1" s="1481"/>
-      <x:c r="W1" s="1481"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="1624" t="str">
-        <x:v>Required inside Security Analysis and Selection — not a separate accounting unit</x:v>
+        <x:v>Required for every proposed final holding — concise validation linked to the authoritative Final Scorecards</x:v>
       </x:c>
       <x:c r="B2" s="1624"/>
       <x:c r="C2" s="1624"/>
@@ -14938,12 +14983,10 @@
       <x:c r="S2" s="1624"/>
       <x:c r="T2" s="1624"/>
       <x:c r="U2" s="1624"/>
-      <x:c r="V2" s="1624"/>
-      <x:c r="W2" s="1624"/>
-    </x:row>
-    <x:row r="4" ht="40" customHeight="1">
+    </x:row>
+    <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="1628" t="str">
-        <x:v>DECISION RULE — Yield or recent return alone cannot support a recommendation. Evidence the issuer's financial health, operating outlook, and relevance to the client's mandate.</x:v>
+        <x:v>DECISION RULE — Validate what each proposed holding owns or represents, how it changes the portfolio, and whether current evidence supports its allocation. Recent return or headline yield cannot substitute for exposure, fit, and risk analysis.</x:v>
       </x:c>
       <x:c r="B4" s="1628"/>
       <x:c r="C4" s="1628"/>
@@ -14965,12 +15008,10 @@
       <x:c r="S4" s="1628"/>
       <x:c r="T4" s="1628"/>
       <x:c r="U4" s="1628"/>
-      <x:c r="V4" s="1628"/>
-      <x:c r="W4" s="1628"/>
-    </x:row>
-    <x:row r="5" ht="34" customHeight="1">
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="1589" t="str">
-        <x:v>APPLIES TO — Every direct individual security. For a selected fund or ETF, complete look-through issuer analysis only when one holding is material to the exposure, concentration, or risk conclusion; do not duplicate the final-holding scorecard.</x:v>
+        <x:v>FUNDS / ETFs FIRST — Review fund or security exposure and strategy; holdings, sector, and style overlap or concentration; costs and liquidity where relevant; key risk; client fit; allocation implication; and current sources. Do not perform company-style financial-health analysis for funds or ETFs.</x:v>
       </x:c>
       <x:c r="B5" s="1589"/>
       <x:c r="C5" s="1589"/>
@@ -14992,12 +15033,10 @@
       <x:c r="S5" s="1589"/>
       <x:c r="T5" s="1589"/>
       <x:c r="U5" s="1589"/>
-      <x:c r="V5" s="1589"/>
-      <x:c r="W5" s="1589"/>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="1485" t="str">
-        <x:v>ROLE HANDOFF — Fixed-Income: duration/credit/income  |  Equity: equity funds/ETFs and limited individual equities  |  Client &amp; Macro: mandate/scenario fit  |  Portfolio Manager: final selection/weights/trade-offs  |  Risk &amp; Derivatives: stress and residual risk</x:v>
+        <x:v>CONDITIONAL DIRECT-SECURITY ADD-ON — Only when the team selects one of the limited direct individual securities, add its material business or issuer-specific risk and the rationale supporting its position size.</x:v>
       </x:c>
       <x:c r="B7" s="1485"/>
       <x:c r="C7" s="1485"/>
@@ -15019,12 +15058,10 @@
       <x:c r="S7" s="1485"/>
       <x:c r="T7" s="1485"/>
       <x:c r="U7" s="1485"/>
-      <x:c r="V7" s="1485"/>
-      <x:c r="W7" s="1485"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="1632" t="str">
-        <x:v>EXPOSURE &amp; EVIDENCE</x:v>
+        <x:v>HOLDING &amp; EXPOSURE</x:v>
       </x:c>
       <x:c r="B9" s="1632"/>
       <x:c r="C9" s="1632"/>
@@ -15034,39 +15071,37 @@
       <x:c r="G9" s="1632"/>
       <x:c r="H9" s="1632"/>
       <x:c r="I9" s="1636" t="str">
-        <x:v>ISSUER HEALTH &amp; OUTLOOK</x:v>
+        <x:v>PORTFOLIO FIT &amp; IMPLEMENTATION</x:v>
       </x:c>
       <x:c r="J9" s="1636"/>
       <x:c r="K9" s="1636"/>
       <x:c r="L9" s="1636"/>
       <x:c r="M9" s="1636"/>
       <x:c r="N9" s="1636"/>
-      <x:c r="O9" s="1636"/>
-      <x:c r="P9" s="1636"/>
-      <x:c r="Q9" s="1636"/>
-      <x:c r="R9" s="1640" t="str">
-        <x:v>RISK, CLIENT FIT &amp; ALLOCATION</x:v>
-      </x:c>
+      <x:c r="O9" s="1640" t="str">
+        <x:v>EVIDENCE &amp; CONDITIONAL DIRECT-SECURITY ADD-ON</x:v>
+      </x:c>
+      <x:c r="P9" s="1640"/>
+      <x:c r="Q9" s="1640"/>
+      <x:c r="R9" s="1640"/>
       <x:c r="S9" s="1640"/>
-      <x:c r="T9" s="1640"/>
-      <x:c r="U9" s="1640"/>
-      <x:c r="V9" s="1644" t="str">
+      <x:c r="T9" s="1644" t="str">
         <x:v>REVIEW</x:v>
       </x:c>
-      <x:c r="W9" s="1644"/>
-    </x:row>
-    <x:row r="10" ht="58" customHeight="1">
+      <x:c r="U9" s="1644"/>
+    </x:row>
+    <x:row r="10" ht="66" customHeight="1">
       <x:c r="A10" s="1655" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="B10" s="1656" t="str">
-        <x:v>Exposure Type</x:v>
+        <x:v>Slot</x:v>
       </x:c>
       <x:c r="C10" s="1656" t="str">
-        <x:v>Security / Fund</x:v>
+        <x:v>Proposed Final Holding</x:v>
       </x:c>
       <x:c r="D10" s="1656" t="str">
-        <x:v>Issuer / Look-Through Holding</x:v>
+        <x:v>Holding Type</x:v>
       </x:c>
       <x:c r="E10" s="1656" t="str">
         <x:v>Portfolio Weight</x:v>
@@ -15075,66 +15110,74 @@
         <x:v>Primary Owner</x:v>
       </x:c>
       <x:c r="G10" s="1656" t="str">
+        <x:v>Fund / Security Exposure &amp; Strategy</x:v>
+      </x:c>
+      <x:c r="H10" s="1656" t="str">
+        <x:v>Holdings / Sector / Style</x:v>
+      </x:c>
+      <x:c r="I10" s="1656" t="str">
+        <x:v>Overlap / Concentration Conclusion</x:v>
+      </x:c>
+      <x:c r="J10" s="1656" t="str">
+        <x:v>Cost &amp; Trading Expenses</x:v>
+      </x:c>
+      <x:c r="K10" s="1656" t="str">
+        <x:v>Liquidity</x:v>
+      </x:c>
+      <x:c r="L10" s="1656" t="str">
+        <x:v>Key Risk</x:v>
+      </x:c>
+      <x:c r="M10" s="1656" t="str">
+        <x:v>Client-Mandate Fit</x:v>
+      </x:c>
+      <x:c r="N10" s="1656" t="str">
+        <x:v>Allocation Implication</x:v>
+      </x:c>
+      <x:c r="O10" s="1656" t="str">
         <x:v>Source / URL</x:v>
       </x:c>
-      <x:c r="H10" s="1656" t="str">
+      <x:c r="P10" s="1656" t="str">
         <x:v>As-of Date</x:v>
       </x:c>
-      <x:c r="I10" s="1656" t="str">
-        <x:v>Business Model</x:v>
-      </x:c>
-      <x:c r="J10" s="1656" t="str">
-        <x:v>Revenue Drivers</x:v>
-      </x:c>
-      <x:c r="K10" s="1656" t="str">
-        <x:v>Industry / Macro Sensitivity</x:v>
-      </x:c>
-      <x:c r="L10" s="1656" t="str">
-        <x:v>Revenue Trend</x:v>
-      </x:c>
-      <x:c r="M10" s="1656" t="str">
-        <x:v>Margin Trend</x:v>
-      </x:c>
-      <x:c r="N10" s="1656" t="str">
-        <x:v>Cash-Flow Trend</x:v>
-      </x:c>
-      <x:c r="O10" s="1656" t="str">
-        <x:v>Liquidity</x:v>
-      </x:c>
-      <x:c r="P10" s="1656" t="str">
-        <x:v>Leverage</x:v>
-      </x:c>
       <x:c r="Q10" s="1656" t="str">
-        <x:v>Interest Coverage / Debt Maturities (if relevant)</x:v>
+        <x:v>Direct-Security Business / Issuer-Specific Risk (if selected)</x:v>
       </x:c>
       <x:c r="R10" s="1656" t="str">
-        <x:v>Issuer-Specific Risk</x:v>
+        <x:v>Direct-Security Position-Size Rationale (if selected)</x:v>
       </x:c>
       <x:c r="S10" s="1656" t="str">
-        <x:v>Client-Fit Conclusion</x:v>
+        <x:v>Monitoring Trigger</x:v>
       </x:c>
       <x:c r="T10" s="1656" t="str">
-        <x:v>Allocation Implication</x:v>
-      </x:c>
-      <x:c r="U10" s="1656" t="str">
-        <x:v>Monitoring Trigger</x:v>
-      </x:c>
-      <x:c r="V10" s="1656" t="str">
         <x:v>Peer Reviewer</x:v>
       </x:c>
-      <x:c r="W10" s="1657" t="str">
+      <x:c r="U10" s="1657" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="64" customHeight="1">
-      <x:c r="A11" s="1685"/>
-      <x:c r="B11" s="1686"/>
-      <x:c r="C11" s="1686"/>
-      <x:c r="D11" s="1686"/>
-      <x:c r="E11" s="1697"/>
-      <x:c r="F11" s="1686"/>
-      <x:c r="G11" s="1686"/>
-      <x:c r="H11" s="1700"/>
+    <x:row r="11" ht="68" customHeight="1">
+      <x:c r="A11" s="1697" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A6="","",'FINAL SCORECARDS'!A6)</x:f>
+        <x:v>Client 1</x:v>
+      </x:c>
+      <x:c r="B11" s="1698" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B6="","",'FINAL SCORECARDS'!B6)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C11" s="1698" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C6="","",'FINAL SCORECARDS'!C6)</x:f>
+      </x:c>
+      <x:c r="D11" s="1698" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D6="","",'FINAL SCORECARDS'!D6)</x:f>
+      </x:c>
+      <x:c r="E11" s="1709" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G6="","",'FINAL SCORECARDS'!G6)</x:f>
+      </x:c>
+      <x:c r="F11" s="1699" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E6="","",'FINAL SCORECARDS'!E6)</x:f>
+      </x:c>
+      <x:c r="G11" s="1677"/>
+      <x:c r="H11" s="1677"/>
       <x:c r="I11" s="1677"/>
       <x:c r="J11" s="1677"/>
       <x:c r="K11" s="1677"/>
@@ -15142,24 +15185,36 @@
       <x:c r="M11" s="1677"/>
       <x:c r="N11" s="1677"/>
       <x:c r="O11" s="1677"/>
-      <x:c r="P11" s="1677"/>
+      <x:c r="P11" s="1711"/>
       <x:c r="Q11" s="1677"/>
       <x:c r="R11" s="1677"/>
       <x:c r="S11" s="1677"/>
-      <x:c r="T11" s="1677"/>
-      <x:c r="U11" s="1677"/>
-      <x:c r="V11" s="1691"/>
-      <x:c r="W11" s="1692"/>
-    </x:row>
-    <x:row r="12" ht="64" customHeight="1">
-      <x:c r="A12" s="1687"/>
-      <x:c r="B12" s="1688"/>
-      <x:c r="C12" s="1688"/>
-      <x:c r="D12" s="1688"/>
-      <x:c r="E12" s="1698"/>
-      <x:c r="F12" s="1688"/>
-      <x:c r="G12" s="1688"/>
-      <x:c r="H12" s="1701"/>
+      <x:c r="T11" s="1703"/>
+      <x:c r="U11" s="1704"/>
+    </x:row>
+    <x:row r="12" ht="68" customHeight="1">
+      <x:c r="A12" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A7="","",'FINAL SCORECARDS'!A7)</x:f>
+        <x:v>Client 1</x:v>
+      </x:c>
+      <x:c r="B12" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B7="","",'FINAL SCORECARDS'!B7)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C12" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C7="","",'FINAL SCORECARDS'!C7)</x:f>
+      </x:c>
+      <x:c r="D12" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D7="","",'FINAL SCORECARDS'!D7)</x:f>
+      </x:c>
+      <x:c r="E12" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G7="","",'FINAL SCORECARDS'!G7)</x:f>
+      </x:c>
+      <x:c r="F12" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E7="","",'FINAL SCORECARDS'!E7)</x:f>
+      </x:c>
+      <x:c r="G12" s="1680"/>
+      <x:c r="H12" s="1680"/>
       <x:c r="I12" s="1680"/>
       <x:c r="J12" s="1680"/>
       <x:c r="K12" s="1680"/>
@@ -15167,24 +15222,36 @@
       <x:c r="M12" s="1680"/>
       <x:c r="N12" s="1680"/>
       <x:c r="O12" s="1680"/>
-      <x:c r="P12" s="1680"/>
+      <x:c r="P12" s="1712"/>
       <x:c r="Q12" s="1680"/>
       <x:c r="R12" s="1680"/>
       <x:c r="S12" s="1680"/>
-      <x:c r="T12" s="1680"/>
-      <x:c r="U12" s="1680"/>
-      <x:c r="V12" s="1693"/>
-      <x:c r="W12" s="1694"/>
-    </x:row>
-    <x:row r="13" ht="64" customHeight="1">
-      <x:c r="A13" s="1687"/>
-      <x:c r="B13" s="1688"/>
-      <x:c r="C13" s="1688"/>
-      <x:c r="D13" s="1688"/>
-      <x:c r="E13" s="1698"/>
-      <x:c r="F13" s="1688"/>
-      <x:c r="G13" s="1688"/>
-      <x:c r="H13" s="1701"/>
+      <x:c r="T12" s="1705"/>
+      <x:c r="U12" s="1706"/>
+    </x:row>
+    <x:row r="13" ht="68" customHeight="1">
+      <x:c r="A13" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A8="","",'FINAL SCORECARDS'!A8)</x:f>
+        <x:v>Client 1</x:v>
+      </x:c>
+      <x:c r="B13" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B8="","",'FINAL SCORECARDS'!B8)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C13" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C8="","",'FINAL SCORECARDS'!C8)</x:f>
+      </x:c>
+      <x:c r="D13" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D8="","",'FINAL SCORECARDS'!D8)</x:f>
+      </x:c>
+      <x:c r="E13" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G8="","",'FINAL SCORECARDS'!G8)</x:f>
+      </x:c>
+      <x:c r="F13" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E8="","",'FINAL SCORECARDS'!E8)</x:f>
+      </x:c>
+      <x:c r="G13" s="1680"/>
+      <x:c r="H13" s="1680"/>
       <x:c r="I13" s="1680"/>
       <x:c r="J13" s="1680"/>
       <x:c r="K13" s="1680"/>
@@ -15192,24 +15259,36 @@
       <x:c r="M13" s="1680"/>
       <x:c r="N13" s="1680"/>
       <x:c r="O13" s="1680"/>
-      <x:c r="P13" s="1680"/>
+      <x:c r="P13" s="1712"/>
       <x:c r="Q13" s="1680"/>
       <x:c r="R13" s="1680"/>
       <x:c r="S13" s="1680"/>
-      <x:c r="T13" s="1680"/>
-      <x:c r="U13" s="1680"/>
-      <x:c r="V13" s="1693"/>
-      <x:c r="W13" s="1694"/>
-    </x:row>
-    <x:row r="14" ht="64" customHeight="1">
-      <x:c r="A14" s="1687"/>
-      <x:c r="B14" s="1688"/>
-      <x:c r="C14" s="1688"/>
-      <x:c r="D14" s="1688"/>
-      <x:c r="E14" s="1698"/>
-      <x:c r="F14" s="1688"/>
-      <x:c r="G14" s="1688"/>
-      <x:c r="H14" s="1701"/>
+      <x:c r="T13" s="1705"/>
+      <x:c r="U13" s="1706"/>
+    </x:row>
+    <x:row r="14" ht="68" customHeight="1">
+      <x:c r="A14" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A9="","",'FINAL SCORECARDS'!A9)</x:f>
+        <x:v>Client 1</x:v>
+      </x:c>
+      <x:c r="B14" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B9="","",'FINAL SCORECARDS'!B9)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C14" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C9="","",'FINAL SCORECARDS'!C9)</x:f>
+      </x:c>
+      <x:c r="D14" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D9="","",'FINAL SCORECARDS'!D9)</x:f>
+      </x:c>
+      <x:c r="E14" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G9="","",'FINAL SCORECARDS'!G9)</x:f>
+      </x:c>
+      <x:c r="F14" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E9="","",'FINAL SCORECARDS'!E9)</x:f>
+      </x:c>
+      <x:c r="G14" s="1680"/>
+      <x:c r="H14" s="1680"/>
       <x:c r="I14" s="1680"/>
       <x:c r="J14" s="1680"/>
       <x:c r="K14" s="1680"/>
@@ -15217,24 +15296,36 @@
       <x:c r="M14" s="1680"/>
       <x:c r="N14" s="1680"/>
       <x:c r="O14" s="1680"/>
-      <x:c r="P14" s="1680"/>
+      <x:c r="P14" s="1712"/>
       <x:c r="Q14" s="1680"/>
       <x:c r="R14" s="1680"/>
       <x:c r="S14" s="1680"/>
-      <x:c r="T14" s="1680"/>
-      <x:c r="U14" s="1680"/>
-      <x:c r="V14" s="1693"/>
-      <x:c r="W14" s="1694"/>
-    </x:row>
-    <x:row r="15" ht="64" customHeight="1">
-      <x:c r="A15" s="1687"/>
-      <x:c r="B15" s="1688"/>
-      <x:c r="C15" s="1688"/>
-      <x:c r="D15" s="1688"/>
-      <x:c r="E15" s="1698"/>
-      <x:c r="F15" s="1688"/>
-      <x:c r="G15" s="1688"/>
-      <x:c r="H15" s="1701"/>
+      <x:c r="T14" s="1705"/>
+      <x:c r="U14" s="1706"/>
+    </x:row>
+    <x:row r="15" ht="68" customHeight="1">
+      <x:c r="A15" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A10="","",'FINAL SCORECARDS'!A10)</x:f>
+        <x:v>Client 1</x:v>
+      </x:c>
+      <x:c r="B15" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B10="","",'FINAL SCORECARDS'!B10)</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C15" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C10="","",'FINAL SCORECARDS'!C10)</x:f>
+      </x:c>
+      <x:c r="D15" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D10="","",'FINAL SCORECARDS'!D10)</x:f>
+      </x:c>
+      <x:c r="E15" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G10="","",'FINAL SCORECARDS'!G10)</x:f>
+      </x:c>
+      <x:c r="F15" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E10="","",'FINAL SCORECARDS'!E10)</x:f>
+      </x:c>
+      <x:c r="G15" s="1680"/>
+      <x:c r="H15" s="1680"/>
       <x:c r="I15" s="1680"/>
       <x:c r="J15" s="1680"/>
       <x:c r="K15" s="1680"/>
@@ -15242,24 +15333,36 @@
       <x:c r="M15" s="1680"/>
       <x:c r="N15" s="1680"/>
       <x:c r="O15" s="1680"/>
-      <x:c r="P15" s="1680"/>
+      <x:c r="P15" s="1712"/>
       <x:c r="Q15" s="1680"/>
       <x:c r="R15" s="1680"/>
       <x:c r="S15" s="1680"/>
-      <x:c r="T15" s="1680"/>
-      <x:c r="U15" s="1680"/>
-      <x:c r="V15" s="1693"/>
-      <x:c r="W15" s="1694"/>
-    </x:row>
-    <x:row r="16" ht="64" customHeight="1">
-      <x:c r="A16" s="1687"/>
-      <x:c r="B16" s="1688"/>
-      <x:c r="C16" s="1688"/>
-      <x:c r="D16" s="1688"/>
-      <x:c r="E16" s="1698"/>
-      <x:c r="F16" s="1688"/>
-      <x:c r="G16" s="1688"/>
-      <x:c r="H16" s="1701"/>
+      <x:c r="T15" s="1705"/>
+      <x:c r="U15" s="1706"/>
+    </x:row>
+    <x:row r="16" ht="68" customHeight="1">
+      <x:c r="A16" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A11="","",'FINAL SCORECARDS'!A11)</x:f>
+        <x:v>Client 1</x:v>
+      </x:c>
+      <x:c r="B16" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B11="","",'FINAL SCORECARDS'!B11)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C16" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C11="","",'FINAL SCORECARDS'!C11)</x:f>
+      </x:c>
+      <x:c r="D16" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D11="","",'FINAL SCORECARDS'!D11)</x:f>
+      </x:c>
+      <x:c r="E16" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G11="","",'FINAL SCORECARDS'!G11)</x:f>
+      </x:c>
+      <x:c r="F16" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E11="","",'FINAL SCORECARDS'!E11)</x:f>
+      </x:c>
+      <x:c r="G16" s="1680"/>
+      <x:c r="H16" s="1680"/>
       <x:c r="I16" s="1680"/>
       <x:c r="J16" s="1680"/>
       <x:c r="K16" s="1680"/>
@@ -15267,24 +15370,36 @@
       <x:c r="M16" s="1680"/>
       <x:c r="N16" s="1680"/>
       <x:c r="O16" s="1680"/>
-      <x:c r="P16" s="1680"/>
+      <x:c r="P16" s="1712"/>
       <x:c r="Q16" s="1680"/>
       <x:c r="R16" s="1680"/>
       <x:c r="S16" s="1680"/>
-      <x:c r="T16" s="1680"/>
-      <x:c r="U16" s="1680"/>
-      <x:c r="V16" s="1693"/>
-      <x:c r="W16" s="1694"/>
-    </x:row>
-    <x:row r="17" ht="64" customHeight="1">
-      <x:c r="A17" s="1687"/>
-      <x:c r="B17" s="1688"/>
-      <x:c r="C17" s="1688"/>
-      <x:c r="D17" s="1688"/>
-      <x:c r="E17" s="1698"/>
-      <x:c r="F17" s="1688"/>
-      <x:c r="G17" s="1688"/>
-      <x:c r="H17" s="1701"/>
+      <x:c r="T16" s="1705"/>
+      <x:c r="U16" s="1706"/>
+    </x:row>
+    <x:row r="17" ht="68" customHeight="1">
+      <x:c r="A17" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A12="","",'FINAL SCORECARDS'!A12)</x:f>
+        <x:v>Client 1</x:v>
+      </x:c>
+      <x:c r="B17" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B12="","",'FINAL SCORECARDS'!B12)</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C17" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C12="","",'FINAL SCORECARDS'!C12)</x:f>
+      </x:c>
+      <x:c r="D17" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D12="","",'FINAL SCORECARDS'!D12)</x:f>
+      </x:c>
+      <x:c r="E17" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G12="","",'FINAL SCORECARDS'!G12)</x:f>
+      </x:c>
+      <x:c r="F17" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E12="","",'FINAL SCORECARDS'!E12)</x:f>
+      </x:c>
+      <x:c r="G17" s="1680"/>
+      <x:c r="H17" s="1680"/>
       <x:c r="I17" s="1680"/>
       <x:c r="J17" s="1680"/>
       <x:c r="K17" s="1680"/>
@@ -15292,24 +15407,36 @@
       <x:c r="M17" s="1680"/>
       <x:c r="N17" s="1680"/>
       <x:c r="O17" s="1680"/>
-      <x:c r="P17" s="1680"/>
+      <x:c r="P17" s="1712"/>
       <x:c r="Q17" s="1680"/>
       <x:c r="R17" s="1680"/>
       <x:c r="S17" s="1680"/>
-      <x:c r="T17" s="1680"/>
-      <x:c r="U17" s="1680"/>
-      <x:c r="V17" s="1693"/>
-      <x:c r="W17" s="1694"/>
-    </x:row>
-    <x:row r="18" ht="64" customHeight="1">
-      <x:c r="A18" s="1687"/>
-      <x:c r="B18" s="1688"/>
-      <x:c r="C18" s="1688"/>
-      <x:c r="D18" s="1688"/>
-      <x:c r="E18" s="1698"/>
-      <x:c r="F18" s="1688"/>
-      <x:c r="G18" s="1688"/>
-      <x:c r="H18" s="1701"/>
+      <x:c r="T17" s="1705"/>
+      <x:c r="U17" s="1706"/>
+    </x:row>
+    <x:row r="18" ht="68" customHeight="1">
+      <x:c r="A18" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A13="","",'FINAL SCORECARDS'!A13)</x:f>
+        <x:v>Client 1</x:v>
+      </x:c>
+      <x:c r="B18" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B13="","",'FINAL SCORECARDS'!B13)</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C18" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C13="","",'FINAL SCORECARDS'!C13)</x:f>
+      </x:c>
+      <x:c r="D18" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D13="","",'FINAL SCORECARDS'!D13)</x:f>
+      </x:c>
+      <x:c r="E18" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G13="","",'FINAL SCORECARDS'!G13)</x:f>
+      </x:c>
+      <x:c r="F18" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E13="","",'FINAL SCORECARDS'!E13)</x:f>
+      </x:c>
+      <x:c r="G18" s="1680"/>
+      <x:c r="H18" s="1680"/>
       <x:c r="I18" s="1680"/>
       <x:c r="J18" s="1680"/>
       <x:c r="K18" s="1680"/>
@@ -15317,24 +15444,36 @@
       <x:c r="M18" s="1680"/>
       <x:c r="N18" s="1680"/>
       <x:c r="O18" s="1680"/>
-      <x:c r="P18" s="1680"/>
+      <x:c r="P18" s="1712"/>
       <x:c r="Q18" s="1680"/>
       <x:c r="R18" s="1680"/>
       <x:c r="S18" s="1680"/>
-      <x:c r="T18" s="1680"/>
-      <x:c r="U18" s="1680"/>
-      <x:c r="V18" s="1693"/>
-      <x:c r="W18" s="1694"/>
-    </x:row>
-    <x:row r="19" ht="64" customHeight="1">
-      <x:c r="A19" s="1687"/>
-      <x:c r="B19" s="1688"/>
-      <x:c r="C19" s="1688"/>
-      <x:c r="D19" s="1688"/>
-      <x:c r="E19" s="1698"/>
-      <x:c r="F19" s="1688"/>
-      <x:c r="G19" s="1688"/>
-      <x:c r="H19" s="1701"/>
+      <x:c r="T18" s="1705"/>
+      <x:c r="U18" s="1706"/>
+    </x:row>
+    <x:row r="19" ht="68" customHeight="1">
+      <x:c r="A19" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A14="","",'FINAL SCORECARDS'!A14)</x:f>
+        <x:v>Client 1</x:v>
+      </x:c>
+      <x:c r="B19" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B14="","",'FINAL SCORECARDS'!B14)</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C19" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C14="","",'FINAL SCORECARDS'!C14)</x:f>
+      </x:c>
+      <x:c r="D19" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D14="","",'FINAL SCORECARDS'!D14)</x:f>
+      </x:c>
+      <x:c r="E19" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G14="","",'FINAL SCORECARDS'!G14)</x:f>
+      </x:c>
+      <x:c r="F19" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E14="","",'FINAL SCORECARDS'!E14)</x:f>
+      </x:c>
+      <x:c r="G19" s="1680"/>
+      <x:c r="H19" s="1680"/>
       <x:c r="I19" s="1680"/>
       <x:c r="J19" s="1680"/>
       <x:c r="K19" s="1680"/>
@@ -15342,24 +15481,36 @@
       <x:c r="M19" s="1680"/>
       <x:c r="N19" s="1680"/>
       <x:c r="O19" s="1680"/>
-      <x:c r="P19" s="1680"/>
+      <x:c r="P19" s="1712"/>
       <x:c r="Q19" s="1680"/>
       <x:c r="R19" s="1680"/>
       <x:c r="S19" s="1680"/>
-      <x:c r="T19" s="1680"/>
-      <x:c r="U19" s="1680"/>
-      <x:c r="V19" s="1693"/>
-      <x:c r="W19" s="1694"/>
-    </x:row>
-    <x:row r="20" ht="64" customHeight="1">
-      <x:c r="A20" s="1687"/>
-      <x:c r="B20" s="1688"/>
-      <x:c r="C20" s="1688"/>
-      <x:c r="D20" s="1688"/>
-      <x:c r="E20" s="1698"/>
-      <x:c r="F20" s="1688"/>
-      <x:c r="G20" s="1688"/>
-      <x:c r="H20" s="1701"/>
+      <x:c r="T19" s="1705"/>
+      <x:c r="U19" s="1706"/>
+    </x:row>
+    <x:row r="20" ht="68" customHeight="1">
+      <x:c r="A20" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A15="","",'FINAL SCORECARDS'!A15)</x:f>
+        <x:v>Client 1</x:v>
+      </x:c>
+      <x:c r="B20" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B15="","",'FINAL SCORECARDS'!B15)</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C20" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C15="","",'FINAL SCORECARDS'!C15)</x:f>
+      </x:c>
+      <x:c r="D20" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D15="","",'FINAL SCORECARDS'!D15)</x:f>
+      </x:c>
+      <x:c r="E20" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G15="","",'FINAL SCORECARDS'!G15)</x:f>
+      </x:c>
+      <x:c r="F20" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E15="","",'FINAL SCORECARDS'!E15)</x:f>
+      </x:c>
+      <x:c r="G20" s="1680"/>
+      <x:c r="H20" s="1680"/>
       <x:c r="I20" s="1680"/>
       <x:c r="J20" s="1680"/>
       <x:c r="K20" s="1680"/>
@@ -15367,24 +15518,36 @@
       <x:c r="M20" s="1680"/>
       <x:c r="N20" s="1680"/>
       <x:c r="O20" s="1680"/>
-      <x:c r="P20" s="1680"/>
+      <x:c r="P20" s="1712"/>
       <x:c r="Q20" s="1680"/>
       <x:c r="R20" s="1680"/>
       <x:c r="S20" s="1680"/>
-      <x:c r="T20" s="1680"/>
-      <x:c r="U20" s="1680"/>
-      <x:c r="V20" s="1693"/>
-      <x:c r="W20" s="1694"/>
-    </x:row>
-    <x:row r="21" ht="64" customHeight="1">
-      <x:c r="A21" s="1687"/>
-      <x:c r="B21" s="1688"/>
-      <x:c r="C21" s="1688"/>
-      <x:c r="D21" s="1688"/>
-      <x:c r="E21" s="1698"/>
-      <x:c r="F21" s="1688"/>
-      <x:c r="G21" s="1688"/>
-      <x:c r="H21" s="1701"/>
+      <x:c r="T20" s="1705"/>
+      <x:c r="U20" s="1706"/>
+    </x:row>
+    <x:row r="21" ht="68" customHeight="1">
+      <x:c r="A21" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A16="","",'FINAL SCORECARDS'!A16)</x:f>
+        <x:v>Client 2</x:v>
+      </x:c>
+      <x:c r="B21" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B16="","",'FINAL SCORECARDS'!B16)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C21" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C16="","",'FINAL SCORECARDS'!C16)</x:f>
+      </x:c>
+      <x:c r="D21" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D16="","",'FINAL SCORECARDS'!D16)</x:f>
+      </x:c>
+      <x:c r="E21" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G16="","",'FINAL SCORECARDS'!G16)</x:f>
+      </x:c>
+      <x:c r="F21" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E16="","",'FINAL SCORECARDS'!E16)</x:f>
+      </x:c>
+      <x:c r="G21" s="1680"/>
+      <x:c r="H21" s="1680"/>
       <x:c r="I21" s="1680"/>
       <x:c r="J21" s="1680"/>
       <x:c r="K21" s="1680"/>
@@ -15392,88 +15555,756 @@
       <x:c r="M21" s="1680"/>
       <x:c r="N21" s="1680"/>
       <x:c r="O21" s="1680"/>
-      <x:c r="P21" s="1680"/>
+      <x:c r="P21" s="1712"/>
       <x:c r="Q21" s="1680"/>
       <x:c r="R21" s="1680"/>
       <x:c r="S21" s="1680"/>
-      <x:c r="T21" s="1680"/>
-      <x:c r="U21" s="1680"/>
-      <x:c r="V21" s="1693"/>
-      <x:c r="W21" s="1694"/>
-    </x:row>
-    <x:row r="22" ht="64" customHeight="1">
-      <x:c r="A22" s="1689"/>
-      <x:c r="B22" s="1690"/>
-      <x:c r="C22" s="1690"/>
-      <x:c r="D22" s="1690"/>
-      <x:c r="E22" s="1699"/>
-      <x:c r="F22" s="1690"/>
-      <x:c r="G22" s="1690"/>
-      <x:c r="H22" s="1702"/>
-      <x:c r="I22" s="1683"/>
-      <x:c r="J22" s="1683"/>
-      <x:c r="K22" s="1683"/>
-      <x:c r="L22" s="1683"/>
-      <x:c r="M22" s="1683"/>
-      <x:c r="N22" s="1683"/>
-      <x:c r="O22" s="1683"/>
-      <x:c r="P22" s="1683"/>
-      <x:c r="Q22" s="1683"/>
-      <x:c r="R22" s="1683"/>
-      <x:c r="S22" s="1683"/>
-      <x:c r="T22" s="1683"/>
-      <x:c r="U22" s="1683"/>
-      <x:c r="V22" s="1695"/>
-      <x:c r="W22" s="1696"/>
-    </x:row>
-    <x:row r="24" ht="40" customHeight="1">
-      <x:c r="A24" s="1706" t="str">
-        <x:v>COMPLETION STANDARD — Concise and cited. Show consistent financial periods, label missing information, and end with a client-fit and allocation conclusion. A second team member reviews each row before committee approval.</x:v>
-      </x:c>
-      <x:c r="B24" s="1706"/>
-      <x:c r="C24" s="1706"/>
-      <x:c r="D24" s="1706"/>
-      <x:c r="E24" s="1706"/>
-      <x:c r="F24" s="1706"/>
-      <x:c r="G24" s="1706"/>
-      <x:c r="H24" s="1706"/>
-      <x:c r="I24" s="1706"/>
-      <x:c r="J24" s="1706"/>
-      <x:c r="K24" s="1706"/>
-      <x:c r="L24" s="1706"/>
-      <x:c r="M24" s="1706"/>
-      <x:c r="N24" s="1706"/>
-      <x:c r="O24" s="1706"/>
-      <x:c r="P24" s="1706"/>
-      <x:c r="Q24" s="1706"/>
-      <x:c r="R24" s="1706"/>
-      <x:c r="S24" s="1706"/>
-      <x:c r="T24" s="1706"/>
+      <x:c r="T21" s="1705"/>
+      <x:c r="U21" s="1706"/>
+    </x:row>
+    <x:row r="22" ht="68" customHeight="1">
+      <x:c r="A22" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A17="","",'FINAL SCORECARDS'!A17)</x:f>
+        <x:v>Client 2</x:v>
+      </x:c>
+      <x:c r="B22" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B17="","",'FINAL SCORECARDS'!B17)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C22" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C17="","",'FINAL SCORECARDS'!C17)</x:f>
+      </x:c>
+      <x:c r="D22" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D17="","",'FINAL SCORECARDS'!D17)</x:f>
+      </x:c>
+      <x:c r="E22" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G17="","",'FINAL SCORECARDS'!G17)</x:f>
+      </x:c>
+      <x:c r="F22" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E17="","",'FINAL SCORECARDS'!E17)</x:f>
+      </x:c>
+      <x:c r="G22" s="1680"/>
+      <x:c r="H22" s="1680"/>
+      <x:c r="I22" s="1680"/>
+      <x:c r="J22" s="1680"/>
+      <x:c r="K22" s="1680"/>
+      <x:c r="L22" s="1680"/>
+      <x:c r="M22" s="1680"/>
+      <x:c r="N22" s="1680"/>
+      <x:c r="O22" s="1680"/>
+      <x:c r="P22" s="1712"/>
+      <x:c r="Q22" s="1680"/>
+      <x:c r="R22" s="1680"/>
+      <x:c r="S22" s="1680"/>
+      <x:c r="T22" s="1705"/>
+      <x:c r="U22" s="1706"/>
+    </x:row>
+    <x:row r="23" ht="68" customHeight="1">
+      <x:c r="A23" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A18="","",'FINAL SCORECARDS'!A18)</x:f>
+        <x:v>Client 2</x:v>
+      </x:c>
+      <x:c r="B23" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B18="","",'FINAL SCORECARDS'!B18)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C23" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C18="","",'FINAL SCORECARDS'!C18)</x:f>
+      </x:c>
+      <x:c r="D23" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D18="","",'FINAL SCORECARDS'!D18)</x:f>
+      </x:c>
+      <x:c r="E23" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G18="","",'FINAL SCORECARDS'!G18)</x:f>
+      </x:c>
+      <x:c r="F23" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E18="","",'FINAL SCORECARDS'!E18)</x:f>
+      </x:c>
+      <x:c r="G23" s="1680"/>
+      <x:c r="H23" s="1680"/>
+      <x:c r="I23" s="1680"/>
+      <x:c r="J23" s="1680"/>
+      <x:c r="K23" s="1680"/>
+      <x:c r="L23" s="1680"/>
+      <x:c r="M23" s="1680"/>
+      <x:c r="N23" s="1680"/>
+      <x:c r="O23" s="1680"/>
+      <x:c r="P23" s="1712"/>
+      <x:c r="Q23" s="1680"/>
+      <x:c r="R23" s="1680"/>
+      <x:c r="S23" s="1680"/>
+      <x:c r="T23" s="1705"/>
+      <x:c r="U23" s="1706"/>
+    </x:row>
+    <x:row r="24" ht="68" customHeight="1">
+      <x:c r="A24" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A19="","",'FINAL SCORECARDS'!A19)</x:f>
+        <x:v>Client 2</x:v>
+      </x:c>
+      <x:c r="B24" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B19="","",'FINAL SCORECARDS'!B19)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C24" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C19="","",'FINAL SCORECARDS'!C19)</x:f>
+      </x:c>
+      <x:c r="D24" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D19="","",'FINAL SCORECARDS'!D19)</x:f>
+      </x:c>
+      <x:c r="E24" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G19="","",'FINAL SCORECARDS'!G19)</x:f>
+      </x:c>
+      <x:c r="F24" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E19="","",'FINAL SCORECARDS'!E19)</x:f>
+      </x:c>
+      <x:c r="G24" s="1680"/>
+      <x:c r="H24" s="1680"/>
+      <x:c r="I24" s="1680"/>
+      <x:c r="J24" s="1680"/>
+      <x:c r="K24" s="1680"/>
+      <x:c r="L24" s="1680"/>
+      <x:c r="M24" s="1680"/>
+      <x:c r="N24" s="1680"/>
+      <x:c r="O24" s="1680"/>
+      <x:c r="P24" s="1712"/>
+      <x:c r="Q24" s="1680"/>
+      <x:c r="R24" s="1680"/>
+      <x:c r="S24" s="1680"/>
+      <x:c r="T24" s="1705"/>
       <x:c r="U24" s="1706"/>
-      <x:c r="V24" s="1706"/>
-      <x:c r="W24" s="1706"/>
+    </x:row>
+    <x:row r="25" ht="68" customHeight="1">
+      <x:c r="A25" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A20="","",'FINAL SCORECARDS'!A20)</x:f>
+        <x:v>Client 2</x:v>
+      </x:c>
+      <x:c r="B25" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B20="","",'FINAL SCORECARDS'!B20)</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C25" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C20="","",'FINAL SCORECARDS'!C20)</x:f>
+      </x:c>
+      <x:c r="D25" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D20="","",'FINAL SCORECARDS'!D20)</x:f>
+      </x:c>
+      <x:c r="E25" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G20="","",'FINAL SCORECARDS'!G20)</x:f>
+      </x:c>
+      <x:c r="F25" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E20="","",'FINAL SCORECARDS'!E20)</x:f>
+      </x:c>
+      <x:c r="G25" s="1680"/>
+      <x:c r="H25" s="1680"/>
+      <x:c r="I25" s="1680"/>
+      <x:c r="J25" s="1680"/>
+      <x:c r="K25" s="1680"/>
+      <x:c r="L25" s="1680"/>
+      <x:c r="M25" s="1680"/>
+      <x:c r="N25" s="1680"/>
+      <x:c r="O25" s="1680"/>
+      <x:c r="P25" s="1712"/>
+      <x:c r="Q25" s="1680"/>
+      <x:c r="R25" s="1680"/>
+      <x:c r="S25" s="1680"/>
+      <x:c r="T25" s="1705"/>
+      <x:c r="U25" s="1706"/>
+    </x:row>
+    <x:row r="26" ht="68" customHeight="1">
+      <x:c r="A26" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A21="","",'FINAL SCORECARDS'!A21)</x:f>
+        <x:v>Client 2</x:v>
+      </x:c>
+      <x:c r="B26" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B21="","",'FINAL SCORECARDS'!B21)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C26" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C21="","",'FINAL SCORECARDS'!C21)</x:f>
+      </x:c>
+      <x:c r="D26" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D21="","",'FINAL SCORECARDS'!D21)</x:f>
+      </x:c>
+      <x:c r="E26" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G21="","",'FINAL SCORECARDS'!G21)</x:f>
+      </x:c>
+      <x:c r="F26" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E21="","",'FINAL SCORECARDS'!E21)</x:f>
+      </x:c>
+      <x:c r="G26" s="1680"/>
+      <x:c r="H26" s="1680"/>
+      <x:c r="I26" s="1680"/>
+      <x:c r="J26" s="1680"/>
+      <x:c r="K26" s="1680"/>
+      <x:c r="L26" s="1680"/>
+      <x:c r="M26" s="1680"/>
+      <x:c r="N26" s="1680"/>
+      <x:c r="O26" s="1680"/>
+      <x:c r="P26" s="1712"/>
+      <x:c r="Q26" s="1680"/>
+      <x:c r="R26" s="1680"/>
+      <x:c r="S26" s="1680"/>
+      <x:c r="T26" s="1705"/>
+      <x:c r="U26" s="1706"/>
+    </x:row>
+    <x:row r="27" ht="68" customHeight="1">
+      <x:c r="A27" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A22="","",'FINAL SCORECARDS'!A22)</x:f>
+        <x:v>Client 2</x:v>
+      </x:c>
+      <x:c r="B27" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B22="","",'FINAL SCORECARDS'!B22)</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C27" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C22="","",'FINAL SCORECARDS'!C22)</x:f>
+      </x:c>
+      <x:c r="D27" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D22="","",'FINAL SCORECARDS'!D22)</x:f>
+      </x:c>
+      <x:c r="E27" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G22="","",'FINAL SCORECARDS'!G22)</x:f>
+      </x:c>
+      <x:c r="F27" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E22="","",'FINAL SCORECARDS'!E22)</x:f>
+      </x:c>
+      <x:c r="G27" s="1680"/>
+      <x:c r="H27" s="1680"/>
+      <x:c r="I27" s="1680"/>
+      <x:c r="J27" s="1680"/>
+      <x:c r="K27" s="1680"/>
+      <x:c r="L27" s="1680"/>
+      <x:c r="M27" s="1680"/>
+      <x:c r="N27" s="1680"/>
+      <x:c r="O27" s="1680"/>
+      <x:c r="P27" s="1712"/>
+      <x:c r="Q27" s="1680"/>
+      <x:c r="R27" s="1680"/>
+      <x:c r="S27" s="1680"/>
+      <x:c r="T27" s="1705"/>
+      <x:c r="U27" s="1706"/>
+    </x:row>
+    <x:row r="28" ht="68" customHeight="1">
+      <x:c r="A28" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A23="","",'FINAL SCORECARDS'!A23)</x:f>
+        <x:v>Client 2</x:v>
+      </x:c>
+      <x:c r="B28" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B23="","",'FINAL SCORECARDS'!B23)</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C28" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C23="","",'FINAL SCORECARDS'!C23)</x:f>
+      </x:c>
+      <x:c r="D28" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D23="","",'FINAL SCORECARDS'!D23)</x:f>
+      </x:c>
+      <x:c r="E28" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G23="","",'FINAL SCORECARDS'!G23)</x:f>
+      </x:c>
+      <x:c r="F28" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E23="","",'FINAL SCORECARDS'!E23)</x:f>
+      </x:c>
+      <x:c r="G28" s="1680"/>
+      <x:c r="H28" s="1680"/>
+      <x:c r="I28" s="1680"/>
+      <x:c r="J28" s="1680"/>
+      <x:c r="K28" s="1680"/>
+      <x:c r="L28" s="1680"/>
+      <x:c r="M28" s="1680"/>
+      <x:c r="N28" s="1680"/>
+      <x:c r="O28" s="1680"/>
+      <x:c r="P28" s="1712"/>
+      <x:c r="Q28" s="1680"/>
+      <x:c r="R28" s="1680"/>
+      <x:c r="S28" s="1680"/>
+      <x:c r="T28" s="1705"/>
+      <x:c r="U28" s="1706"/>
+    </x:row>
+    <x:row r="29" ht="68" customHeight="1">
+      <x:c r="A29" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A24="","",'FINAL SCORECARDS'!A24)</x:f>
+        <x:v>Client 2</x:v>
+      </x:c>
+      <x:c r="B29" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B24="","",'FINAL SCORECARDS'!B24)</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C29" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C24="","",'FINAL SCORECARDS'!C24)</x:f>
+      </x:c>
+      <x:c r="D29" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D24="","",'FINAL SCORECARDS'!D24)</x:f>
+      </x:c>
+      <x:c r="E29" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G24="","",'FINAL SCORECARDS'!G24)</x:f>
+      </x:c>
+      <x:c r="F29" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E24="","",'FINAL SCORECARDS'!E24)</x:f>
+      </x:c>
+      <x:c r="G29" s="1680"/>
+      <x:c r="H29" s="1680"/>
+      <x:c r="I29" s="1680"/>
+      <x:c r="J29" s="1680"/>
+      <x:c r="K29" s="1680"/>
+      <x:c r="L29" s="1680"/>
+      <x:c r="M29" s="1680"/>
+      <x:c r="N29" s="1680"/>
+      <x:c r="O29" s="1680"/>
+      <x:c r="P29" s="1712"/>
+      <x:c r="Q29" s="1680"/>
+      <x:c r="R29" s="1680"/>
+      <x:c r="S29" s="1680"/>
+      <x:c r="T29" s="1705"/>
+      <x:c r="U29" s="1706"/>
+    </x:row>
+    <x:row r="30" ht="68" customHeight="1">
+      <x:c r="A30" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A25="","",'FINAL SCORECARDS'!A25)</x:f>
+        <x:v>Client 2</x:v>
+      </x:c>
+      <x:c r="B30" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B25="","",'FINAL SCORECARDS'!B25)</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C30" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C25="","",'FINAL SCORECARDS'!C25)</x:f>
+      </x:c>
+      <x:c r="D30" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D25="","",'FINAL SCORECARDS'!D25)</x:f>
+      </x:c>
+      <x:c r="E30" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G25="","",'FINAL SCORECARDS'!G25)</x:f>
+      </x:c>
+      <x:c r="F30" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E25="","",'FINAL SCORECARDS'!E25)</x:f>
+      </x:c>
+      <x:c r="G30" s="1680"/>
+      <x:c r="H30" s="1680"/>
+      <x:c r="I30" s="1680"/>
+      <x:c r="J30" s="1680"/>
+      <x:c r="K30" s="1680"/>
+      <x:c r="L30" s="1680"/>
+      <x:c r="M30" s="1680"/>
+      <x:c r="N30" s="1680"/>
+      <x:c r="O30" s="1680"/>
+      <x:c r="P30" s="1712"/>
+      <x:c r="Q30" s="1680"/>
+      <x:c r="R30" s="1680"/>
+      <x:c r="S30" s="1680"/>
+      <x:c r="T30" s="1705"/>
+      <x:c r="U30" s="1706"/>
+    </x:row>
+    <x:row r="31" ht="68" customHeight="1">
+      <x:c r="A31" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A26="","",'FINAL SCORECARDS'!A26)</x:f>
+        <x:v>Client 3</x:v>
+      </x:c>
+      <x:c r="B31" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B26="","",'FINAL SCORECARDS'!B26)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C31" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C26="","",'FINAL SCORECARDS'!C26)</x:f>
+      </x:c>
+      <x:c r="D31" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D26="","",'FINAL SCORECARDS'!D26)</x:f>
+      </x:c>
+      <x:c r="E31" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G26="","",'FINAL SCORECARDS'!G26)</x:f>
+      </x:c>
+      <x:c r="F31" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E26="","",'FINAL SCORECARDS'!E26)</x:f>
+      </x:c>
+      <x:c r="G31" s="1680"/>
+      <x:c r="H31" s="1680"/>
+      <x:c r="I31" s="1680"/>
+      <x:c r="J31" s="1680"/>
+      <x:c r="K31" s="1680"/>
+      <x:c r="L31" s="1680"/>
+      <x:c r="M31" s="1680"/>
+      <x:c r="N31" s="1680"/>
+      <x:c r="O31" s="1680"/>
+      <x:c r="P31" s="1712"/>
+      <x:c r="Q31" s="1680"/>
+      <x:c r="R31" s="1680"/>
+      <x:c r="S31" s="1680"/>
+      <x:c r="T31" s="1705"/>
+      <x:c r="U31" s="1706"/>
+    </x:row>
+    <x:row r="32" ht="68" customHeight="1">
+      <x:c r="A32" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A27="","",'FINAL SCORECARDS'!A27)</x:f>
+        <x:v>Client 3</x:v>
+      </x:c>
+      <x:c r="B32" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B27="","",'FINAL SCORECARDS'!B27)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C32" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C27="","",'FINAL SCORECARDS'!C27)</x:f>
+      </x:c>
+      <x:c r="D32" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D27="","",'FINAL SCORECARDS'!D27)</x:f>
+      </x:c>
+      <x:c r="E32" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G27="","",'FINAL SCORECARDS'!G27)</x:f>
+      </x:c>
+      <x:c r="F32" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E27="","",'FINAL SCORECARDS'!E27)</x:f>
+      </x:c>
+      <x:c r="G32" s="1680"/>
+      <x:c r="H32" s="1680"/>
+      <x:c r="I32" s="1680"/>
+      <x:c r="J32" s="1680"/>
+      <x:c r="K32" s="1680"/>
+      <x:c r="L32" s="1680"/>
+      <x:c r="M32" s="1680"/>
+      <x:c r="N32" s="1680"/>
+      <x:c r="O32" s="1680"/>
+      <x:c r="P32" s="1712"/>
+      <x:c r="Q32" s="1680"/>
+      <x:c r="R32" s="1680"/>
+      <x:c r="S32" s="1680"/>
+      <x:c r="T32" s="1705"/>
+      <x:c r="U32" s="1706"/>
+    </x:row>
+    <x:row r="33" ht="68" customHeight="1">
+      <x:c r="A33" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A28="","",'FINAL SCORECARDS'!A28)</x:f>
+        <x:v>Client 3</x:v>
+      </x:c>
+      <x:c r="B33" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B28="","",'FINAL SCORECARDS'!B28)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C33" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C28="","",'FINAL SCORECARDS'!C28)</x:f>
+      </x:c>
+      <x:c r="D33" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D28="","",'FINAL SCORECARDS'!D28)</x:f>
+      </x:c>
+      <x:c r="E33" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G28="","",'FINAL SCORECARDS'!G28)</x:f>
+      </x:c>
+      <x:c r="F33" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E28="","",'FINAL SCORECARDS'!E28)</x:f>
+      </x:c>
+      <x:c r="G33" s="1680"/>
+      <x:c r="H33" s="1680"/>
+      <x:c r="I33" s="1680"/>
+      <x:c r="J33" s="1680"/>
+      <x:c r="K33" s="1680"/>
+      <x:c r="L33" s="1680"/>
+      <x:c r="M33" s="1680"/>
+      <x:c r="N33" s="1680"/>
+      <x:c r="O33" s="1680"/>
+      <x:c r="P33" s="1712"/>
+      <x:c r="Q33" s="1680"/>
+      <x:c r="R33" s="1680"/>
+      <x:c r="S33" s="1680"/>
+      <x:c r="T33" s="1705"/>
+      <x:c r="U33" s="1706"/>
+    </x:row>
+    <x:row r="34" ht="68" customHeight="1">
+      <x:c r="A34" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A29="","",'FINAL SCORECARDS'!A29)</x:f>
+        <x:v>Client 3</x:v>
+      </x:c>
+      <x:c r="B34" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B29="","",'FINAL SCORECARDS'!B29)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C34" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C29="","",'FINAL SCORECARDS'!C29)</x:f>
+      </x:c>
+      <x:c r="D34" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D29="","",'FINAL SCORECARDS'!D29)</x:f>
+      </x:c>
+      <x:c r="E34" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G29="","",'FINAL SCORECARDS'!G29)</x:f>
+      </x:c>
+      <x:c r="F34" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E29="","",'FINAL SCORECARDS'!E29)</x:f>
+      </x:c>
+      <x:c r="G34" s="1680"/>
+      <x:c r="H34" s="1680"/>
+      <x:c r="I34" s="1680"/>
+      <x:c r="J34" s="1680"/>
+      <x:c r="K34" s="1680"/>
+      <x:c r="L34" s="1680"/>
+      <x:c r="M34" s="1680"/>
+      <x:c r="N34" s="1680"/>
+      <x:c r="O34" s="1680"/>
+      <x:c r="P34" s="1712"/>
+      <x:c r="Q34" s="1680"/>
+      <x:c r="R34" s="1680"/>
+      <x:c r="S34" s="1680"/>
+      <x:c r="T34" s="1705"/>
+      <x:c r="U34" s="1706"/>
+    </x:row>
+    <x:row r="35" ht="68" customHeight="1">
+      <x:c r="A35" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A30="","",'FINAL SCORECARDS'!A30)</x:f>
+        <x:v>Client 3</x:v>
+      </x:c>
+      <x:c r="B35" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B30="","",'FINAL SCORECARDS'!B30)</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C35" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C30="","",'FINAL SCORECARDS'!C30)</x:f>
+      </x:c>
+      <x:c r="D35" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D30="","",'FINAL SCORECARDS'!D30)</x:f>
+      </x:c>
+      <x:c r="E35" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G30="","",'FINAL SCORECARDS'!G30)</x:f>
+      </x:c>
+      <x:c r="F35" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E30="","",'FINAL SCORECARDS'!E30)</x:f>
+      </x:c>
+      <x:c r="G35" s="1680"/>
+      <x:c r="H35" s="1680"/>
+      <x:c r="I35" s="1680"/>
+      <x:c r="J35" s="1680"/>
+      <x:c r="K35" s="1680"/>
+      <x:c r="L35" s="1680"/>
+      <x:c r="M35" s="1680"/>
+      <x:c r="N35" s="1680"/>
+      <x:c r="O35" s="1680"/>
+      <x:c r="P35" s="1712"/>
+      <x:c r="Q35" s="1680"/>
+      <x:c r="R35" s="1680"/>
+      <x:c r="S35" s="1680"/>
+      <x:c r="T35" s="1705"/>
+      <x:c r="U35" s="1706"/>
+    </x:row>
+    <x:row r="36" ht="68" customHeight="1">
+      <x:c r="A36" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A31="","",'FINAL SCORECARDS'!A31)</x:f>
+        <x:v>Client 3</x:v>
+      </x:c>
+      <x:c r="B36" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B31="","",'FINAL SCORECARDS'!B31)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C36" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C31="","",'FINAL SCORECARDS'!C31)</x:f>
+      </x:c>
+      <x:c r="D36" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D31="","",'FINAL SCORECARDS'!D31)</x:f>
+      </x:c>
+      <x:c r="E36" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G31="","",'FINAL SCORECARDS'!G31)</x:f>
+      </x:c>
+      <x:c r="F36" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E31="","",'FINAL SCORECARDS'!E31)</x:f>
+      </x:c>
+      <x:c r="G36" s="1680"/>
+      <x:c r="H36" s="1680"/>
+      <x:c r="I36" s="1680"/>
+      <x:c r="J36" s="1680"/>
+      <x:c r="K36" s="1680"/>
+      <x:c r="L36" s="1680"/>
+      <x:c r="M36" s="1680"/>
+      <x:c r="N36" s="1680"/>
+      <x:c r="O36" s="1680"/>
+      <x:c r="P36" s="1712"/>
+      <x:c r="Q36" s="1680"/>
+      <x:c r="R36" s="1680"/>
+      <x:c r="S36" s="1680"/>
+      <x:c r="T36" s="1705"/>
+      <x:c r="U36" s="1706"/>
+    </x:row>
+    <x:row r="37" ht="68" customHeight="1">
+      <x:c r="A37" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A32="","",'FINAL SCORECARDS'!A32)</x:f>
+        <x:v>Client 3</x:v>
+      </x:c>
+      <x:c r="B37" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B32="","",'FINAL SCORECARDS'!B32)</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C37" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C32="","",'FINAL SCORECARDS'!C32)</x:f>
+      </x:c>
+      <x:c r="D37" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D32="","",'FINAL SCORECARDS'!D32)</x:f>
+      </x:c>
+      <x:c r="E37" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G32="","",'FINAL SCORECARDS'!G32)</x:f>
+      </x:c>
+      <x:c r="F37" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E32="","",'FINAL SCORECARDS'!E32)</x:f>
+      </x:c>
+      <x:c r="G37" s="1680"/>
+      <x:c r="H37" s="1680"/>
+      <x:c r="I37" s="1680"/>
+      <x:c r="J37" s="1680"/>
+      <x:c r="K37" s="1680"/>
+      <x:c r="L37" s="1680"/>
+      <x:c r="M37" s="1680"/>
+      <x:c r="N37" s="1680"/>
+      <x:c r="O37" s="1680"/>
+      <x:c r="P37" s="1712"/>
+      <x:c r="Q37" s="1680"/>
+      <x:c r="R37" s="1680"/>
+      <x:c r="S37" s="1680"/>
+      <x:c r="T37" s="1705"/>
+      <x:c r="U37" s="1706"/>
+    </x:row>
+    <x:row r="38" ht="68" customHeight="1">
+      <x:c r="A38" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A33="","",'FINAL SCORECARDS'!A33)</x:f>
+        <x:v>Client 3</x:v>
+      </x:c>
+      <x:c r="B38" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B33="","",'FINAL SCORECARDS'!B33)</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C38" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C33="","",'FINAL SCORECARDS'!C33)</x:f>
+      </x:c>
+      <x:c r="D38" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D33="","",'FINAL SCORECARDS'!D33)</x:f>
+      </x:c>
+      <x:c r="E38" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G33="","",'FINAL SCORECARDS'!G33)</x:f>
+      </x:c>
+      <x:c r="F38" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E33="","",'FINAL SCORECARDS'!E33)</x:f>
+      </x:c>
+      <x:c r="G38" s="1680"/>
+      <x:c r="H38" s="1680"/>
+      <x:c r="I38" s="1680"/>
+      <x:c r="J38" s="1680"/>
+      <x:c r="K38" s="1680"/>
+      <x:c r="L38" s="1680"/>
+      <x:c r="M38" s="1680"/>
+      <x:c r="N38" s="1680"/>
+      <x:c r="O38" s="1680"/>
+      <x:c r="P38" s="1712"/>
+      <x:c r="Q38" s="1680"/>
+      <x:c r="R38" s="1680"/>
+      <x:c r="S38" s="1680"/>
+      <x:c r="T38" s="1705"/>
+      <x:c r="U38" s="1706"/>
+    </x:row>
+    <x:row r="39" ht="68" customHeight="1">
+      <x:c r="A39" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A34="","",'FINAL SCORECARDS'!A34)</x:f>
+        <x:v>Client 3</x:v>
+      </x:c>
+      <x:c r="B39" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B34="","",'FINAL SCORECARDS'!B34)</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C39" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C34="","",'FINAL SCORECARDS'!C34)</x:f>
+      </x:c>
+      <x:c r="D39" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D34="","",'FINAL SCORECARDS'!D34)</x:f>
+      </x:c>
+      <x:c r="E39" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G34="","",'FINAL SCORECARDS'!G34)</x:f>
+      </x:c>
+      <x:c r="F39" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E34="","",'FINAL SCORECARDS'!E34)</x:f>
+      </x:c>
+      <x:c r="G39" s="1680"/>
+      <x:c r="H39" s="1680"/>
+      <x:c r="I39" s="1680"/>
+      <x:c r="J39" s="1680"/>
+      <x:c r="K39" s="1680"/>
+      <x:c r="L39" s="1680"/>
+      <x:c r="M39" s="1680"/>
+      <x:c r="N39" s="1680"/>
+      <x:c r="O39" s="1680"/>
+      <x:c r="P39" s="1712"/>
+      <x:c r="Q39" s="1680"/>
+      <x:c r="R39" s="1680"/>
+      <x:c r="S39" s="1680"/>
+      <x:c r="T39" s="1705"/>
+      <x:c r="U39" s="1706"/>
+    </x:row>
+    <x:row r="40" ht="68" customHeight="1">
+      <x:c r="A40" s="1700" t="str">
+        <x:f>IF('FINAL SCORECARDS'!A35="","",'FINAL SCORECARDS'!A35)</x:f>
+        <x:v>Client 3</x:v>
+      </x:c>
+      <x:c r="B40" s="1701" t="n">
+        <x:f>IF('FINAL SCORECARDS'!B35="","",'FINAL SCORECARDS'!B35)</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C40" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!C35="","",'FINAL SCORECARDS'!C35)</x:f>
+      </x:c>
+      <x:c r="D40" s="1701" t="str">
+        <x:f>IF('FINAL SCORECARDS'!D35="","",'FINAL SCORECARDS'!D35)</x:f>
+      </x:c>
+      <x:c r="E40" s="1710" t="str">
+        <x:f>IF('FINAL SCORECARDS'!G35="","",'FINAL SCORECARDS'!G35)</x:f>
+      </x:c>
+      <x:c r="F40" s="1702" t="str">
+        <x:f>IF('FINAL SCORECARDS'!E35="","",'FINAL SCORECARDS'!E35)</x:f>
+      </x:c>
+      <x:c r="G40" s="1683"/>
+      <x:c r="H40" s="1683"/>
+      <x:c r="I40" s="1683"/>
+      <x:c r="J40" s="1683"/>
+      <x:c r="K40" s="1683"/>
+      <x:c r="L40" s="1683"/>
+      <x:c r="M40" s="1683"/>
+      <x:c r="N40" s="1683"/>
+      <x:c r="O40" s="1683"/>
+      <x:c r="P40" s="1713"/>
+      <x:c r="Q40" s="1683"/>
+      <x:c r="R40" s="1683"/>
+      <x:c r="S40" s="1683"/>
+      <x:c r="T40" s="1707"/>
+      <x:c r="U40" s="1708"/>
+    </x:row>
+    <x:row r="42" ht="48" customHeight="1">
+      <x:c r="A42" s="1717" t="str">
+        <x:v>COMPLETION STANDARD — One concise row per proposed final holding, linked to FINAL SCORECARDS. Funds and ETFs require exposure, overlap/concentration, implementation, risk, fit, allocation, and source evidence—not company-style issuer financials. Complete the two direct-security fields only when applicable. A second team member reviews each row before committee approval.</x:v>
+      </x:c>
+      <x:c r="B42" s="1717"/>
+      <x:c r="C42" s="1717"/>
+      <x:c r="D42" s="1717"/>
+      <x:c r="E42" s="1717"/>
+      <x:c r="F42" s="1717"/>
+      <x:c r="G42" s="1717"/>
+      <x:c r="H42" s="1717"/>
+      <x:c r="I42" s="1717"/>
+      <x:c r="J42" s="1717"/>
+      <x:c r="K42" s="1717"/>
+      <x:c r="L42" s="1717"/>
+      <x:c r="M42" s="1717"/>
+      <x:c r="N42" s="1717"/>
+      <x:c r="O42" s="1717"/>
+      <x:c r="P42" s="1717"/>
+      <x:c r="Q42" s="1717"/>
+      <x:c r="R42" s="1717"/>
+      <x:c r="S42" s="1717"/>
+      <x:c r="T42" s="1717"/>
+      <x:c r="U42" s="1717"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
+    <x:mergeCell ref="A1:U1"/>
+    <x:mergeCell ref="A2:U2"/>
+    <x:mergeCell ref="A4:U4"/>
+    <x:mergeCell ref="A5:U5"/>
+    <x:mergeCell ref="A7:U7"/>
     <x:mergeCell ref="A9:H9"/>
-    <x:mergeCell ref="I9:Q9"/>
-    <x:mergeCell ref="R9:U9"/>
-    <x:mergeCell ref="V9:W9"/>
-    <x:mergeCell ref="A24:W24"/>
-    <x:mergeCell ref="A1:W1"/>
-    <x:mergeCell ref="A2:W2"/>
-    <x:mergeCell ref="A4:W4"/>
-    <x:mergeCell ref="A5:W5"/>
-    <x:mergeCell ref="A7:W7"/>
+    <x:mergeCell ref="I9:N9"/>
+    <x:mergeCell ref="O9:S9"/>
+    <x:mergeCell ref="T9:U9"/>
+    <x:mergeCell ref="A42:U42"/>
   </x:mergeCells>
-  <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="B11:B22">
-      <x:formula1>"Direct bond,Direct equity,Fund/ETF look-through"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="F11:F22">
-      <x:formula1>"Client and Macro Strategist,Fixed-Income Analyst,Equity Analyst,Portfolio Manager,Risk and Derivatives Analyst"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="W11:W22">
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="U11:U40">
       <x:formula1>"Not started,Ready for peer review,Complete,Revise"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -15651,15 +16482,15 @@
       <x:c r="F9" s="1677"/>
       <x:c r="G9" s="1677"/>
       <x:c r="H9" s="1677"/>
-      <x:c r="I9" s="1707"/>
-      <x:c r="J9" s="1707"/>
+      <x:c r="I9" s="1711"/>
+      <x:c r="J9" s="1711"/>
       <x:c r="K9" s="1677"/>
       <x:c r="L9" s="1677"/>
       <x:c r="M9" s="1677"/>
       <x:c r="N9" s="1677"/>
-      <x:c r="O9" s="1691"/>
-      <x:c r="P9" s="1691"/>
-      <x:c r="Q9" s="1692"/>
+      <x:c r="O9" s="1703"/>
+      <x:c r="P9" s="1703"/>
+      <x:c r="Q9" s="1704"/>
     </x:row>
     <x:row r="10" ht="64" customHeight="1">
       <x:c r="A10" s="1687"/>
@@ -15670,15 +16501,15 @@
       <x:c r="F10" s="1680"/>
       <x:c r="G10" s="1680"/>
       <x:c r="H10" s="1680"/>
-      <x:c r="I10" s="1708"/>
-      <x:c r="J10" s="1708"/>
+      <x:c r="I10" s="1712"/>
+      <x:c r="J10" s="1712"/>
       <x:c r="K10" s="1680"/>
       <x:c r="L10" s="1680"/>
       <x:c r="M10" s="1680"/>
       <x:c r="N10" s="1680"/>
-      <x:c r="O10" s="1693"/>
-      <x:c r="P10" s="1693"/>
-      <x:c r="Q10" s="1694"/>
+      <x:c r="O10" s="1705"/>
+      <x:c r="P10" s="1705"/>
+      <x:c r="Q10" s="1706"/>
     </x:row>
     <x:row r="11" ht="64" customHeight="1">
       <x:c r="A11" s="1687"/>
@@ -15689,15 +16520,15 @@
       <x:c r="F11" s="1680"/>
       <x:c r="G11" s="1680"/>
       <x:c r="H11" s="1680"/>
-      <x:c r="I11" s="1708"/>
-      <x:c r="J11" s="1708"/>
+      <x:c r="I11" s="1712"/>
+      <x:c r="J11" s="1712"/>
       <x:c r="K11" s="1680"/>
       <x:c r="L11" s="1680"/>
       <x:c r="M11" s="1680"/>
       <x:c r="N11" s="1680"/>
-      <x:c r="O11" s="1693"/>
-      <x:c r="P11" s="1693"/>
-      <x:c r="Q11" s="1694"/>
+      <x:c r="O11" s="1705"/>
+      <x:c r="P11" s="1705"/>
+      <x:c r="Q11" s="1706"/>
     </x:row>
     <x:row r="12" ht="64" customHeight="1">
       <x:c r="A12" s="1687"/>
@@ -15708,15 +16539,15 @@
       <x:c r="F12" s="1680"/>
       <x:c r="G12" s="1680"/>
       <x:c r="H12" s="1680"/>
-      <x:c r="I12" s="1708"/>
-      <x:c r="J12" s="1708"/>
+      <x:c r="I12" s="1712"/>
+      <x:c r="J12" s="1712"/>
       <x:c r="K12" s="1680"/>
       <x:c r="L12" s="1680"/>
       <x:c r="M12" s="1680"/>
       <x:c r="N12" s="1680"/>
-      <x:c r="O12" s="1693"/>
-      <x:c r="P12" s="1693"/>
-      <x:c r="Q12" s="1694"/>
+      <x:c r="O12" s="1705"/>
+      <x:c r="P12" s="1705"/>
+      <x:c r="Q12" s="1706"/>
     </x:row>
     <x:row r="13" ht="64" customHeight="1">
       <x:c r="A13" s="1687"/>
@@ -15727,15 +16558,15 @@
       <x:c r="F13" s="1680"/>
       <x:c r="G13" s="1680"/>
       <x:c r="H13" s="1680"/>
-      <x:c r="I13" s="1708"/>
-      <x:c r="J13" s="1708"/>
+      <x:c r="I13" s="1712"/>
+      <x:c r="J13" s="1712"/>
       <x:c r="K13" s="1680"/>
       <x:c r="L13" s="1680"/>
       <x:c r="M13" s="1680"/>
       <x:c r="N13" s="1680"/>
-      <x:c r="O13" s="1693"/>
-      <x:c r="P13" s="1693"/>
-      <x:c r="Q13" s="1694"/>
+      <x:c r="O13" s="1705"/>
+      <x:c r="P13" s="1705"/>
+      <x:c r="Q13" s="1706"/>
     </x:row>
     <x:row r="14" ht="64" customHeight="1">
       <x:c r="A14" s="1687"/>
@@ -15746,15 +16577,15 @@
       <x:c r="F14" s="1680"/>
       <x:c r="G14" s="1680"/>
       <x:c r="H14" s="1680"/>
-      <x:c r="I14" s="1708"/>
-      <x:c r="J14" s="1708"/>
+      <x:c r="I14" s="1712"/>
+      <x:c r="J14" s="1712"/>
       <x:c r="K14" s="1680"/>
       <x:c r="L14" s="1680"/>
       <x:c r="M14" s="1680"/>
       <x:c r="N14" s="1680"/>
-      <x:c r="O14" s="1693"/>
-      <x:c r="P14" s="1693"/>
-      <x:c r="Q14" s="1694"/>
+      <x:c r="O14" s="1705"/>
+      <x:c r="P14" s="1705"/>
+      <x:c r="Q14" s="1706"/>
     </x:row>
     <x:row r="15" ht="64" customHeight="1">
       <x:c r="A15" s="1687"/>
@@ -15765,15 +16596,15 @@
       <x:c r="F15" s="1680"/>
       <x:c r="G15" s="1680"/>
       <x:c r="H15" s="1680"/>
-      <x:c r="I15" s="1708"/>
-      <x:c r="J15" s="1708"/>
+      <x:c r="I15" s="1712"/>
+      <x:c r="J15" s="1712"/>
       <x:c r="K15" s="1680"/>
       <x:c r="L15" s="1680"/>
       <x:c r="M15" s="1680"/>
       <x:c r="N15" s="1680"/>
-      <x:c r="O15" s="1693"/>
-      <x:c r="P15" s="1693"/>
-      <x:c r="Q15" s="1694"/>
+      <x:c r="O15" s="1705"/>
+      <x:c r="P15" s="1705"/>
+      <x:c r="Q15" s="1706"/>
     </x:row>
     <x:row r="16" ht="64" customHeight="1">
       <x:c r="A16" s="1687"/>
@@ -15784,15 +16615,15 @@
       <x:c r="F16" s="1680"/>
       <x:c r="G16" s="1680"/>
       <x:c r="H16" s="1680"/>
-      <x:c r="I16" s="1708"/>
-      <x:c r="J16" s="1708"/>
+      <x:c r="I16" s="1712"/>
+      <x:c r="J16" s="1712"/>
       <x:c r="K16" s="1680"/>
       <x:c r="L16" s="1680"/>
       <x:c r="M16" s="1680"/>
       <x:c r="N16" s="1680"/>
-      <x:c r="O16" s="1693"/>
-      <x:c r="P16" s="1693"/>
-      <x:c r="Q16" s="1694"/>
+      <x:c r="O16" s="1705"/>
+      <x:c r="P16" s="1705"/>
+      <x:c r="Q16" s="1706"/>
     </x:row>
     <x:row r="17" ht="64" customHeight="1">
       <x:c r="A17" s="1687"/>
@@ -15803,15 +16634,15 @@
       <x:c r="F17" s="1680"/>
       <x:c r="G17" s="1680"/>
       <x:c r="H17" s="1680"/>
-      <x:c r="I17" s="1708"/>
-      <x:c r="J17" s="1708"/>
+      <x:c r="I17" s="1712"/>
+      <x:c r="J17" s="1712"/>
       <x:c r="K17" s="1680"/>
       <x:c r="L17" s="1680"/>
       <x:c r="M17" s="1680"/>
       <x:c r="N17" s="1680"/>
-      <x:c r="O17" s="1693"/>
-      <x:c r="P17" s="1693"/>
-      <x:c r="Q17" s="1694"/>
+      <x:c r="O17" s="1705"/>
+      <x:c r="P17" s="1705"/>
+      <x:c r="Q17" s="1706"/>
     </x:row>
     <x:row r="18" ht="64" customHeight="1">
       <x:c r="A18" s="1687"/>
@@ -15822,15 +16653,15 @@
       <x:c r="F18" s="1680"/>
       <x:c r="G18" s="1680"/>
       <x:c r="H18" s="1680"/>
-      <x:c r="I18" s="1708"/>
-      <x:c r="J18" s="1708"/>
+      <x:c r="I18" s="1712"/>
+      <x:c r="J18" s="1712"/>
       <x:c r="K18" s="1680"/>
       <x:c r="L18" s="1680"/>
       <x:c r="M18" s="1680"/>
       <x:c r="N18" s="1680"/>
-      <x:c r="O18" s="1693"/>
-      <x:c r="P18" s="1693"/>
-      <x:c r="Q18" s="1694"/>
+      <x:c r="O18" s="1705"/>
+      <x:c r="P18" s="1705"/>
+      <x:c r="Q18" s="1706"/>
     </x:row>
     <x:row r="19" ht="64" customHeight="1">
       <x:c r="A19" s="1687"/>
@@ -15841,15 +16672,15 @@
       <x:c r="F19" s="1680"/>
       <x:c r="G19" s="1680"/>
       <x:c r="H19" s="1680"/>
-      <x:c r="I19" s="1708"/>
-      <x:c r="J19" s="1708"/>
+      <x:c r="I19" s="1712"/>
+      <x:c r="J19" s="1712"/>
       <x:c r="K19" s="1680"/>
       <x:c r="L19" s="1680"/>
       <x:c r="M19" s="1680"/>
       <x:c r="N19" s="1680"/>
-      <x:c r="O19" s="1693"/>
-      <x:c r="P19" s="1693"/>
-      <x:c r="Q19" s="1694"/>
+      <x:c r="O19" s="1705"/>
+      <x:c r="P19" s="1705"/>
+      <x:c r="Q19" s="1706"/>
     </x:row>
     <x:row r="20" ht="64" customHeight="1">
       <x:c r="A20" s="1687"/>
@@ -15860,15 +16691,15 @@
       <x:c r="F20" s="1680"/>
       <x:c r="G20" s="1680"/>
       <x:c r="H20" s="1680"/>
-      <x:c r="I20" s="1708"/>
-      <x:c r="J20" s="1708"/>
+      <x:c r="I20" s="1712"/>
+      <x:c r="J20" s="1712"/>
       <x:c r="K20" s="1680"/>
       <x:c r="L20" s="1680"/>
       <x:c r="M20" s="1680"/>
       <x:c r="N20" s="1680"/>
-      <x:c r="O20" s="1693"/>
-      <x:c r="P20" s="1693"/>
-      <x:c r="Q20" s="1694"/>
+      <x:c r="O20" s="1705"/>
+      <x:c r="P20" s="1705"/>
+      <x:c r="Q20" s="1706"/>
     </x:row>
     <x:row r="21" ht="64" customHeight="1">
       <x:c r="A21" s="1687"/>
@@ -15879,15 +16710,15 @@
       <x:c r="F21" s="1680"/>
       <x:c r="G21" s="1680"/>
       <x:c r="H21" s="1680"/>
-      <x:c r="I21" s="1708"/>
-      <x:c r="J21" s="1708"/>
+      <x:c r="I21" s="1712"/>
+      <x:c r="J21" s="1712"/>
       <x:c r="K21" s="1680"/>
       <x:c r="L21" s="1680"/>
       <x:c r="M21" s="1680"/>
       <x:c r="N21" s="1680"/>
-      <x:c r="O21" s="1693"/>
-      <x:c r="P21" s="1693"/>
-      <x:c r="Q21" s="1694"/>
+      <x:c r="O21" s="1705"/>
+      <x:c r="P21" s="1705"/>
+      <x:c r="Q21" s="1706"/>
     </x:row>
     <x:row r="22" ht="64" customHeight="1">
       <x:c r="A22" s="1687"/>
@@ -15898,15 +16729,15 @@
       <x:c r="F22" s="1680"/>
       <x:c r="G22" s="1680"/>
       <x:c r="H22" s="1680"/>
-      <x:c r="I22" s="1708"/>
-      <x:c r="J22" s="1708"/>
+      <x:c r="I22" s="1712"/>
+      <x:c r="J22" s="1712"/>
       <x:c r="K22" s="1680"/>
       <x:c r="L22" s="1680"/>
       <x:c r="M22" s="1680"/>
       <x:c r="N22" s="1680"/>
-      <x:c r="O22" s="1693"/>
-      <x:c r="P22" s="1693"/>
-      <x:c r="Q22" s="1694"/>
+      <x:c r="O22" s="1705"/>
+      <x:c r="P22" s="1705"/>
+      <x:c r="Q22" s="1706"/>
     </x:row>
     <x:row r="23" ht="64" customHeight="1">
       <x:c r="A23" s="1687"/>
@@ -15917,15 +16748,15 @@
       <x:c r="F23" s="1680"/>
       <x:c r="G23" s="1680"/>
       <x:c r="H23" s="1680"/>
-      <x:c r="I23" s="1708"/>
-      <x:c r="J23" s="1708"/>
+      <x:c r="I23" s="1712"/>
+      <x:c r="J23" s="1712"/>
       <x:c r="K23" s="1680"/>
       <x:c r="L23" s="1680"/>
       <x:c r="M23" s="1680"/>
       <x:c r="N23" s="1680"/>
-      <x:c r="O23" s="1693"/>
-      <x:c r="P23" s="1693"/>
-      <x:c r="Q23" s="1694"/>
+      <x:c r="O23" s="1705"/>
+      <x:c r="P23" s="1705"/>
+      <x:c r="Q23" s="1706"/>
     </x:row>
     <x:row r="24" ht="64" customHeight="1">
       <x:c r="A24" s="1689"/>
@@ -15936,15 +16767,15 @@
       <x:c r="F24" s="1683"/>
       <x:c r="G24" s="1683"/>
       <x:c r="H24" s="1683"/>
-      <x:c r="I24" s="1709"/>
-      <x:c r="J24" s="1709"/>
+      <x:c r="I24" s="1713"/>
+      <x:c r="J24" s="1713"/>
       <x:c r="K24" s="1683"/>
       <x:c r="L24" s="1683"/>
       <x:c r="M24" s="1683"/>
       <x:c r="N24" s="1683"/>
-      <x:c r="O24" s="1695"/>
-      <x:c r="P24" s="1695"/>
-      <x:c r="Q24" s="1696"/>
+      <x:c r="O24" s="1707"/>
+      <x:c r="P24" s="1707"/>
+      <x:c r="Q24" s="1708"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -15955,7 +16786,7 @@
   </x:mergeCells>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B9:B24">
-      <x:formula1>"Issuer Reality Check,Credit / fixed income,Equity fund / ETF,Individual equity,Portfolio integration,Portfolio risk / hedge input"</x:formula1>
+      <x:formula1>"Holding &amp; exposure reality check,Credit / fixed income,Equity fund / ETF,Individual equity,Portfolio integration,Portfolio risk / hedge input"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="L9:L24">
       <x:formula1>"Confirmed,Qualified,Contradicted,Changed,Not verifiable"</x:formula1>
@@ -15989,7 +16820,7 @@
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="1485" t="str">
-        <x:v>Use this guide before completing the client tabs, Issuer Reality Check, and FactSet Research and Evidence Log. It tells you what to investigate; your committee supplies the research, calculations, judgment, and select/reject decision.</x:v>
+        <x:v>Use this guide before completing the client tabs, Final Scorecards, Holding &amp; Exposure Reality Check, and FactSet Research and Evidence Log. It tells you what to investigate; your committee supplies the research, calculations, judgment, and select/reject decision.</x:v>
       </x:c>
       <x:c r="B2" s="1485"/>
       <x:c r="C2" s="1485"/>
@@ -16078,7 +16909,7 @@
         <x:v>Distinct purpose versus a fund/ETF, business and return drivers, liquidity, key risks, client fit, idiosyncratic risk, position-size rationale, concentration limit, and source/as-of date.</x:v>
       </x:c>
       <x:c r="C14" s="1524" t="str">
-        <x:v>Complete the scorecard, Issuer Reality Check, and Evidence Log. Individual securities total no more than two or three per portfolio.</x:v>
+        <x:v>Complete the scorecard, Holding &amp; Exposure Reality Check with its conditional direct-security add-on, and Evidence Log. Direct individual securities total no more than two or three per portfolio.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="104" customHeight="1">

</xml_diff>